<commit_message>
AR24-072: D4 and D5
</commit_message>
<xml_diff>
--- a/data/ar24-072-experiment/AR24-072-SAM-MasterDataTable.xlsx
+++ b/data/ar24-072-experiment/AR24-072-SAM-MasterDataTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myteams.gsk.com/sites/BiopharmModelPredictiveControl/Shared Documents/General/data/AR24-072-SAM-MPC-1kL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2526" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D65E0C2F-8A87-426B-A65C-25FC250267DD}"/>
+  <xr:revisionPtr revIDLastSave="2618" documentId="14_{29998BAB-B97E-4D42-B36C-5857DA37A7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1566A155-7771-4B12-A02E-8311A52F93C1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterDataTable" sheetId="1" r:id="rId1"/>
@@ -314,7 +314,7 @@
     <t>Feed Rate based on CSFR (mL/hr)</t>
   </si>
   <si>
-    <t>Something is wrong with Tech code. Nutrient_rate is too high. MPC underfeeding compared to manual. Cannot manually adjust pumps</t>
+    <t xml:space="preserve"> MPC underfeeding 30%  compared to manual (titer information missing from input file from Tech). Cannot manually adjust pumps. </t>
   </si>
 </sst>
 </file>
@@ -7764,7 +7764,7 @@
         <v>91</v>
       </c>
       <c r="G30" s="83">
-        <v>45570.368055555555</v>
+        <v>45571.368055555555</v>
       </c>
       <c r="H30" s="40">
         <v>1505.08</v>
@@ -8487,7 +8487,7 @@
       </c>
       <c r="AR33" s="42">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>6.2890000000000001E-2</v>
       </c>
       <c r="AS33" s="42">
         <f t="shared" si="23"/>
@@ -8519,7 +8519,9 @@
       <c r="BA33" s="43">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BB33" s="11"/>
+      <c r="BB33" s="11">
+        <v>7.6E-3</v>
+      </c>
       <c r="BC33" s="43"/>
       <c r="BD33" s="22"/>
       <c r="BE33" s="43">
@@ -8544,11 +8546,11 @@
       </c>
       <c r="BJ33" s="44">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>90.561599999999999</v>
       </c>
       <c r="BK33" s="44">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>6.2890000000000001E-2</v>
       </c>
       <c r="BL33" s="44" t="str">
         <f t="shared" si="12"/>
@@ -8568,11 +8570,11 @@
       </c>
       <c r="BP33" s="58">
         <f t="shared" si="41"/>
-        <v>0</v>
+        <v>163.35064935064938</v>
       </c>
       <c r="BQ33" s="46">
         <f t="shared" si="42"/>
-        <v>0</v>
+        <v>6.2890000000000001E-2</v>
       </c>
       <c r="BR33" s="24">
         <f t="shared" si="22"/>
@@ -8703,7 +8705,7 @@
       </c>
       <c r="AR34" s="42">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>0.16416666666666666</v>
       </c>
       <c r="AS34" s="42">
         <f t="shared" si="23"/>
@@ -8735,7 +8737,9 @@
       <c r="BA34" s="43">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BB34" s="11"/>
+      <c r="BB34" s="11">
+        <v>0.02</v>
+      </c>
       <c r="BD34" s="22"/>
       <c r="BE34" s="43">
         <f t="shared" si="1"/>
@@ -8759,11 +8763,11 @@
       </c>
       <c r="BJ34" s="44">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>236.39999999999998</v>
       </c>
       <c r="BK34" s="44">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>0.16416666666666666</v>
       </c>
       <c r="BL34" s="45" t="str">
         <f t="shared" si="12"/>
@@ -8783,11 +8787,11 @@
       </c>
       <c r="BP34" s="58">
         <f t="shared" si="41"/>
-        <v>0</v>
+        <v>426.4069264069264</v>
       </c>
       <c r="BQ34" s="46">
         <f t="shared" si="42"/>
-        <v>0</v>
+        <v>0.16416666666666666</v>
       </c>
       <c r="BR34" s="24">
         <f t="shared" si="22"/>
@@ -8918,7 +8922,7 @@
       </c>
       <c r="AR35" s="42">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>0.12476205211681562</v>
       </c>
       <c r="AS35" s="42">
         <f t="shared" si="23"/>
@@ -8951,7 +8955,14 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BB35" s="11"/>
-      <c r="BD35" s="22"/>
+      <c r="BC35" s="81">
+        <f>0.00207936753528026*24*60/BG35</f>
+        <v>1.5122672983856439E-2</v>
+      </c>
+      <c r="BD35" s="81">
+        <f>0.937837273085801/BG35</f>
+        <v>4.7365518842717221E-3</v>
+      </c>
       <c r="BE35" s="43">
         <f t="shared" ref="BE35:BE66" si="44">BA35*L35*BG35/1000</f>
         <v>1.4315399999999998E-3</v>
@@ -8974,7 +8985,7 @@
       </c>
       <c r="BJ35" s="44">
         <f t="shared" ref="BJ35:BJ66" si="48">AR35*24*60</f>
-        <v>0</v>
+        <v>179.6573550482145</v>
       </c>
       <c r="BK35" s="44" t="str">
         <f t="shared" si="19"/>
@@ -8982,7 +8993,7 @@
       </c>
       <c r="BL35" s="45">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.12476205211681562</v>
       </c>
       <c r="BM35" s="45" t="str">
         <f t="shared" si="13"/>
@@ -8994,19 +9005,19 @@
       </c>
       <c r="BO35" s="44">
         <f t="shared" ref="BO35:BO66" si="49">IF(C35="Julia",BD35*BG35,"")</f>
-        <v>0</v>
+        <v>0.937837273085801</v>
       </c>
       <c r="BP35" s="58">
         <f t="shared" si="41"/>
-        <v>0</v>
+        <v>324.05727822549517</v>
       </c>
       <c r="BQ35" s="46">
         <f t="shared" si="42"/>
-        <v>0</v>
+        <v>0.12476205211681562</v>
       </c>
       <c r="BR35" s="24">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>0.937837273085801</v>
       </c>
     </row>
     <row r="36" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -9133,7 +9144,7 @@
       </c>
       <c r="AR36" s="42">
         <f>BQ36</f>
-        <v>0</v>
+        <v>0.1136403146599332</v>
       </c>
       <c r="AS36" s="42">
         <f t="shared" si="23"/>
@@ -9166,7 +9177,14 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BB36" s="11"/>
-      <c r="BD36" s="22"/>
+      <c r="BC36" s="81">
+        <f>0.00189400524433222*24*60/BG36</f>
+        <v>1.3732968538964737E-2</v>
+      </c>
+      <c r="BD36" s="81">
+        <f>0.950560138745667/BG36</f>
+        <v>4.7863048275209822E-3</v>
+      </c>
       <c r="BE36" s="43">
         <f t="shared" si="44"/>
         <v>1.5192899999999997E-3</v>
@@ -9189,7 +9207,7 @@
       </c>
       <c r="BJ36" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>163.64205311030381</v>
       </c>
       <c r="BK36" s="44" t="str">
         <f t="shared" si="19"/>
@@ -9197,7 +9215,7 @@
       </c>
       <c r="BL36" s="45">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.1136403146599332</v>
       </c>
       <c r="BM36" s="45" t="str">
         <f t="shared" si="13"/>
@@ -9209,19 +9227,19 @@
       </c>
       <c r="BO36" s="44">
         <f t="shared" si="49"/>
-        <v>0</v>
+        <v>0.95056013874566703</v>
       </c>
       <c r="BP36" s="58">
         <f>IF(BK36&lt;&gt;"",BK36/0.000385,IF(BL36&lt;&gt;"",BL36/0.000385,BM36/0.000385))</f>
-        <v>0</v>
+        <v>295.16964846735897</v>
       </c>
       <c r="BQ36" s="46">
         <f>IF(BK36&lt;&gt;"",BK36,IF(BL36&lt;&gt;"",BL36,BM36))</f>
-        <v>0</v>
+        <v>0.1136403146599332</v>
       </c>
       <c r="BR36" s="24">
         <f>IF(BN36&lt;&gt;"",BN36,BO36)</f>
-        <v>0</v>
+        <v>0.95056013874566703</v>
       </c>
     </row>
     <row r="37" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -9671,24 +9689,38 @@
         <v>4</v>
       </c>
       <c r="F39" s="3"/>
-      <c r="G39" s="34"/>
+      <c r="G39" s="34">
+        <v>45572.359027777777</v>
+      </c>
       <c r="H39" s="3">
         <v>2119.61</v>
       </c>
       <c r="I39" s="6"/>
-      <c r="J39" s="6"/>
-      <c r="K39" s="6"/>
-      <c r="L39" s="6"/>
-      <c r="M39" s="6"/>
+      <c r="J39" s="6">
+        <v>1588.47</v>
+      </c>
+      <c r="K39" s="6">
+        <v>21.1</v>
+      </c>
+      <c r="L39" s="6">
+        <v>20.8</v>
+      </c>
+      <c r="M39" s="6">
+        <v>98.3</v>
+      </c>
       <c r="N39" s="6"/>
       <c r="O39" s="6"/>
       <c r="P39" s="6"/>
       <c r="Q39" s="6"/>
-      <c r="R39" s="6"/>
+      <c r="R39" s="6">
+        <v>1.76</v>
+      </c>
       <c r="S39" s="6"/>
       <c r="T39" s="6"/>
       <c r="U39" s="6"/>
-      <c r="V39" s="6"/>
+      <c r="V39" s="6">
+        <v>2.6</v>
+      </c>
       <c r="W39" s="6"/>
       <c r="X39" s="6"/>
       <c r="Y39" s="6"/>
@@ -9697,33 +9729,45 @@
       <c r="AB39" s="6"/>
       <c r="AC39" s="6"/>
       <c r="AD39" s="6"/>
-      <c r="AE39" s="16"/>
+      <c r="AE39" s="16">
+        <v>7.306</v>
+      </c>
       <c r="AF39" s="6"/>
-      <c r="AG39" s="6"/>
+      <c r="AG39" s="6">
+        <v>50.000105040413999</v>
+      </c>
       <c r="AH39" s="6"/>
-      <c r="AI39" s="6"/>
+      <c r="AI39" s="6">
+        <v>33.997979719765702</v>
+      </c>
       <c r="AJ39" s="6"/>
       <c r="AK39" s="6"/>
       <c r="AL39" s="6"/>
-      <c r="AM39" s="6"/>
-      <c r="AN39" s="6"/>
-      <c r="AO39" s="6"/>
+      <c r="AM39" s="6">
+        <v>22306.763671875</v>
+      </c>
+      <c r="AN39" s="6">
+        <v>14919.5068359375</v>
+      </c>
+      <c r="AO39" s="6">
+        <v>611400</v>
+      </c>
       <c r="AP39" s="72"/>
       <c r="AQ39" s="32">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.50000105040414</v>
       </c>
       <c r="AR39" s="32">
         <f t="shared" ref="AR39:AR70" si="50">BQ39</f>
-        <v>0</v>
+        <v>531.44902002000003</v>
       </c>
       <c r="AS39" s="32">
         <f t="shared" si="23"/>
-        <v>-14699.6376953125</v>
+        <v>7607.1259765625</v>
       </c>
       <c r="AT39" s="32">
         <f t="shared" si="24"/>
-        <v>-10229.482421875</v>
+        <v>4690.0244140625</v>
       </c>
       <c r="AU39" s="32">
         <f t="shared" si="25"/>
@@ -9748,31 +9792,37 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BB39" s="8"/>
-      <c r="BC39" s="9"/>
-      <c r="BD39" s="21"/>
+      <c r="BC39" s="9">
+        <f>8.857483667*24*60/BG39</f>
+        <v>2.0861590579784102E-2</v>
+      </c>
+      <c r="BD39" s="81">
+        <f>2610.0869895953/BG39</f>
+        <v>4.2690333490273142E-3</v>
+      </c>
       <c r="BE39" s="9">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>3.8151359999999999</v>
       </c>
       <c r="BF39" s="9">
         <f t="shared" ref="BF39:BF70" si="51">BE39*24*60</f>
-        <v>0</v>
+        <v>5493.7958400000007</v>
       </c>
       <c r="BG39" s="9">
         <f t="shared" si="45"/>
-        <v>591700</v>
-      </c>
-      <c r="BH39" s="10" t="str">
+        <v>611400</v>
+      </c>
+      <c r="BH39" s="10">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI39" s="10" t="str">
+        <v>3.6484729590897942E-2</v>
+      </c>
+      <c r="BI39" s="10">
         <f t="shared" si="47"/>
-        <v/>
+        <v>3.768034404032939E-2</v>
       </c>
       <c r="BJ39" s="10">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>765286.58882880001</v>
       </c>
       <c r="BK39" s="10" t="str">
         <f t="shared" si="19"/>
@@ -9780,7 +9830,7 @@
       </c>
       <c r="BL39" s="10">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>531.44902002000003</v>
       </c>
       <c r="BM39" s="28" t="str">
         <f t="shared" si="13"/>
@@ -9792,19 +9842,19 @@
       </c>
       <c r="BO39" s="10">
         <f t="shared" si="49"/>
-        <v>0</v>
+        <v>2610.0869895953001</v>
       </c>
       <c r="BP39" s="62">
         <f t="shared" ref="BP39:BP70" si="52">IF(BK39&lt;&gt;"",BK39/0.000385,IF(BL39&lt;&gt;"",BL39/0.000385,BM39/0.000385))</f>
-        <v>0</v>
+        <v>1380387.0649870131</v>
       </c>
       <c r="BQ39" s="30">
         <f t="shared" ref="BQ39:BQ70" si="53">IF(BK39&lt;&gt;"",BK39,IF(BL39&lt;&gt;"",BL39,BM39))</f>
-        <v>0</v>
+        <v>531.44902002000003</v>
       </c>
       <c r="BR39" s="26">
         <f t="shared" ref="BR39:BR70" si="54">IF(BN39&lt;&gt;"",BN39,BO39)</f>
-        <v>0</v>
+        <v>2610.0869895953001</v>
       </c>
     </row>
     <row r="40" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -9823,59 +9873,123 @@
       <c r="E40" s="40">
         <v>4</v>
       </c>
-      <c r="G40" s="35"/>
+      <c r="G40" s="35">
+        <v>45572.402777777781</v>
+      </c>
       <c r="H40" s="40">
         <v>2119.61</v>
       </c>
       <c r="I40" s="41"/>
-      <c r="J40" s="41"/>
-      <c r="K40" s="41"/>
-      <c r="L40" s="41"/>
-      <c r="M40" s="41"/>
-      <c r="N40" s="41"/>
-      <c r="O40" s="41"/>
-      <c r="P40" s="41"/>
-      <c r="Q40" s="41"/>
-      <c r="R40" s="41"/>
+      <c r="J40" s="41">
+        <v>1786.4549999999999</v>
+      </c>
+      <c r="K40" s="41">
+        <v>25.9</v>
+      </c>
+      <c r="L40" s="41">
+        <v>24.5</v>
+      </c>
+      <c r="M40" s="41">
+        <v>94.7</v>
+      </c>
+      <c r="N40" s="41">
+        <v>16.3</v>
+      </c>
+      <c r="O40" s="41">
+        <v>316</v>
+      </c>
+      <c r="P40" s="41">
+        <v>1.46</v>
+      </c>
+      <c r="Q40" s="41">
+        <v>0.41</v>
+      </c>
+      <c r="R40" s="41">
+        <v>2.14</v>
+      </c>
       <c r="S40" s="41"/>
-      <c r="T40" s="41"/>
-      <c r="U40" s="41"/>
-      <c r="V40" s="41"/>
-      <c r="W40" s="41"/>
-      <c r="X40" s="41"/>
-      <c r="Y40" s="41"/>
-      <c r="Z40" s="41"/>
-      <c r="AA40" s="41"/>
-      <c r="AB40" s="41"/>
-      <c r="AC40" s="41"/>
-      <c r="AD40" s="41"/>
-      <c r="AE40" s="17"/>
-      <c r="AF40" s="41"/>
-      <c r="AG40" s="41"/>
-      <c r="AH40" s="41"/>
-      <c r="AI40" s="41"/>
-      <c r="AJ40" s="41"/>
-      <c r="AK40" s="41"/>
-      <c r="AL40" s="41"/>
-      <c r="AM40" s="41"/>
-      <c r="AN40" s="41"/>
-      <c r="AO40" s="41"/>
+      <c r="T40" s="41">
+        <v>0.13</v>
+      </c>
+      <c r="U40" s="41">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V40" s="41">
+        <v>3.02</v>
+      </c>
+      <c r="W40" s="41">
+        <v>7.2759999999999998</v>
+      </c>
+      <c r="X40" s="41">
+        <v>43.1</v>
+      </c>
+      <c r="Y40" s="41">
+        <v>60.6</v>
+      </c>
+      <c r="Z40" s="41">
+        <v>2.64</v>
+      </c>
+      <c r="AA40" s="41">
+        <v>133.5</v>
+      </c>
+      <c r="AB40" s="41">
+        <v>17.8</v>
+      </c>
+      <c r="AC40" s="41">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="AD40" s="41">
+        <v>49.2</v>
+      </c>
+      <c r="AE40" s="17">
+        <v>7.2359999999999998</v>
+      </c>
+      <c r="AF40" s="41">
+        <v>406</v>
+      </c>
+      <c r="AG40" s="41">
+        <v>52</v>
+      </c>
+      <c r="AH40" s="41">
+        <v>7.3079999999999998</v>
+      </c>
+      <c r="AI40" s="41">
+        <v>33.9</v>
+      </c>
+      <c r="AJ40" s="41">
+        <v>2</v>
+      </c>
+      <c r="AK40" s="41">
+        <v>1.4</v>
+      </c>
+      <c r="AL40" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM40" s="41">
+        <v>6.1</v>
+      </c>
+      <c r="AN40" s="41">
+        <v>4</v>
+      </c>
+      <c r="AO40" s="41">
+        <v>197.4</v>
+      </c>
       <c r="AP40" s="74"/>
       <c r="AQ40" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="AR40" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>8.7053400000000003E-2</v>
       </c>
       <c r="AS40" s="42">
         <f t="shared" si="23"/>
-        <v>-4.2</v>
+        <v>1.8999999999999995</v>
       </c>
       <c r="AT40" s="42">
         <f t="shared" si="24"/>
-        <v>-2.8</v>
+        <v>1.2000000000000002</v>
       </c>
       <c r="AU40" s="42">
         <f t="shared" si="25"/>
@@ -9904,27 +10018,27 @@
       <c r="BD40" s="22"/>
       <c r="BE40" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.45089E-3</v>
       </c>
       <c r="BF40" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.0892816000000001</v>
       </c>
       <c r="BG40" s="43">
         <f t="shared" si="45"/>
-        <v>188</v>
-      </c>
-      <c r="BH40" s="44" t="str">
+        <v>197.4</v>
+      </c>
+      <c r="BH40" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI40" s="44" t="str">
+        <v>3.0901722391084092E-2</v>
+      </c>
+      <c r="BI40" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>3.0499999999999999E-2</v>
       </c>
       <c r="BJ40" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>125.35689600000001</v>
       </c>
       <c r="BK40" s="44" t="str">
         <f t="shared" si="19"/>
@@ -9936,11 +10050,11 @@
       </c>
       <c r="BM40" s="45">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>8.7053400000000003E-2</v>
       </c>
       <c r="BN40" s="44">
         <f t="shared" si="32"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
       <c r="BO40" s="44" t="str">
         <f t="shared" si="49"/>
@@ -9948,15 +10062,15 @@
       </c>
       <c r="BP40" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>226.11272727272728</v>
       </c>
       <c r="BQ40" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>8.7053400000000003E-2</v>
       </c>
       <c r="BR40" s="24">
         <f t="shared" si="54"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -9975,59 +10089,123 @@
       <c r="E41" s="40">
         <v>4</v>
       </c>
-      <c r="G41" s="35"/>
+      <c r="G41" s="35">
+        <v>45572.40347222222</v>
+      </c>
       <c r="H41" s="40">
         <v>2119.61</v>
       </c>
       <c r="I41" s="41"/>
-      <c r="J41" s="41"/>
-      <c r="K41" s="41"/>
-      <c r="L41" s="41"/>
-      <c r="M41" s="41"/>
-      <c r="N41" s="41"/>
-      <c r="O41" s="41"/>
-      <c r="P41" s="41"/>
-      <c r="Q41" s="41"/>
-      <c r="R41" s="41"/>
+      <c r="J41" s="41">
+        <v>1778.8050000000001</v>
+      </c>
+      <c r="K41" s="41">
+        <v>26.8</v>
+      </c>
+      <c r="L41" s="41">
+        <v>25.2</v>
+      </c>
+      <c r="M41" s="41">
+        <v>94.2</v>
+      </c>
+      <c r="N41" s="41">
+        <v>16.2</v>
+      </c>
+      <c r="O41" s="41">
+        <v>319</v>
+      </c>
+      <c r="P41" s="41">
+        <v>1.45</v>
+      </c>
+      <c r="Q41" s="41">
+        <v>0.41</v>
+      </c>
+      <c r="R41" s="41">
+        <v>2.21</v>
+      </c>
       <c r="S41" s="41"/>
-      <c r="T41" s="41"/>
-      <c r="U41" s="41"/>
-      <c r="V41" s="41"/>
-      <c r="W41" s="41"/>
-      <c r="X41" s="41"/>
-      <c r="Y41" s="41"/>
-      <c r="Z41" s="41"/>
-      <c r="AA41" s="41"/>
-      <c r="AB41" s="41"/>
-      <c r="AC41" s="41"/>
-      <c r="AD41" s="41"/>
-      <c r="AE41" s="17"/>
-      <c r="AF41" s="41"/>
-      <c r="AG41" s="41"/>
-      <c r="AH41" s="41"/>
-      <c r="AI41" s="41"/>
-      <c r="AJ41" s="41"/>
-      <c r="AK41" s="41"/>
-      <c r="AL41" s="41"/>
-      <c r="AM41" s="41"/>
-      <c r="AN41" s="41"/>
-      <c r="AO41" s="41"/>
+      <c r="T41" s="41">
+        <v>0.16</v>
+      </c>
+      <c r="U41" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="V41" s="41">
+        <v>3.11</v>
+      </c>
+      <c r="W41" s="41">
+        <v>7.2750000000000004</v>
+      </c>
+      <c r="X41" s="41">
+        <v>45</v>
+      </c>
+      <c r="Y41" s="41">
+        <v>65.400000000000006</v>
+      </c>
+      <c r="Z41" s="41">
+        <v>2.83</v>
+      </c>
+      <c r="AA41" s="41">
+        <v>135.80000000000001</v>
+      </c>
+      <c r="AB41" s="41">
+        <v>18.5</v>
+      </c>
+      <c r="AC41" s="41">
+        <v>39.4</v>
+      </c>
+      <c r="AD41" s="41">
+        <v>53.3</v>
+      </c>
+      <c r="AE41" s="17">
+        <v>7.234</v>
+      </c>
+      <c r="AF41" s="41">
+        <v>406</v>
+      </c>
+      <c r="AG41" s="41">
+        <v>51.1</v>
+      </c>
+      <c r="AH41" s="41">
+        <v>7.3090000000000002</v>
+      </c>
+      <c r="AI41" s="41">
+        <v>33.9</v>
+      </c>
+      <c r="AJ41" s="41">
+        <v>2.1</v>
+      </c>
+      <c r="AK41" s="41">
+        <v>1.2</v>
+      </c>
+      <c r="AL41" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM41" s="41">
+        <v>6</v>
+      </c>
+      <c r="AN41" s="41">
+        <v>4.3</v>
+      </c>
+      <c r="AO41" s="41">
+        <v>197.4</v>
+      </c>
       <c r="AP41" s="74"/>
       <c r="AQ41" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.51100000000000001</v>
       </c>
       <c r="AR41" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>8.9540639999999991E-2</v>
       </c>
       <c r="AS41" s="42">
         <f t="shared" si="23"/>
-        <v>-4</v>
+        <v>2</v>
       </c>
       <c r="AT41" s="42">
         <f t="shared" si="24"/>
-        <v>-3</v>
+        <v>1.2999999999999998</v>
       </c>
       <c r="AU41" s="42">
         <f t="shared" si="25"/>
@@ -10056,27 +10234,27 @@
       <c r="BD41" s="22"/>
       <c r="BE41" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.4923439999999998E-3</v>
       </c>
       <c r="BF41" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.1489753599999997</v>
       </c>
       <c r="BG41" s="43">
         <f t="shared" si="45"/>
-        <v>188</v>
-      </c>
-      <c r="BH41" s="44" t="str">
+        <v>197.4</v>
+      </c>
+      <c r="BH41" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI41" s="44" t="str">
+        <v>3.0395136778115502E-2</v>
+      </c>
+      <c r="BI41" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>0.03</v>
       </c>
       <c r="BJ41" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>128.93852159999997</v>
       </c>
       <c r="BK41" s="44" t="str">
         <f t="shared" si="19"/>
@@ -10088,11 +10266,11 @@
       </c>
       <c r="BM41" s="45">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>8.9540639999999991E-2</v>
       </c>
       <c r="BN41" s="44">
         <f t="shared" si="32"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
       <c r="BO41" s="44" t="str">
         <f t="shared" si="49"/>
@@ -10100,15 +10278,15 @@
       </c>
       <c r="BP41" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>232.57309090909089</v>
       </c>
       <c r="BQ41" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>8.9540639999999991E-2</v>
       </c>
       <c r="BR41" s="24">
         <f t="shared" si="54"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -10127,59 +10305,123 @@
       <c r="E42" s="40">
         <v>4</v>
       </c>
-      <c r="G42" s="35"/>
+      <c r="G42" s="35">
+        <v>45572.404166666667</v>
+      </c>
       <c r="H42" s="40">
         <v>2119.61</v>
       </c>
       <c r="I42" s="41"/>
-      <c r="J42" s="41"/>
-      <c r="K42" s="41"/>
-      <c r="L42" s="41"/>
-      <c r="M42" s="41"/>
-      <c r="N42" s="41"/>
-      <c r="O42" s="41"/>
-      <c r="P42" s="41"/>
-      <c r="Q42" s="41"/>
-      <c r="R42" s="41"/>
+      <c r="J42" s="41">
+        <v>1675.365</v>
+      </c>
+      <c r="K42" s="41">
+        <v>24.8</v>
+      </c>
+      <c r="L42" s="41">
+        <v>22.8</v>
+      </c>
+      <c r="M42" s="41">
+        <v>91.9</v>
+      </c>
+      <c r="N42" s="41">
+        <v>16.7</v>
+      </c>
+      <c r="O42" s="41">
+        <v>350</v>
+      </c>
+      <c r="P42" s="41">
+        <v>2.69</v>
+      </c>
+      <c r="Q42" s="41">
+        <v>0.44</v>
+      </c>
+      <c r="R42" s="41">
+        <v>0.28999999999999998</v>
+      </c>
       <c r="S42" s="41"/>
-      <c r="T42" s="41"/>
-      <c r="U42" s="41"/>
-      <c r="V42" s="41"/>
-      <c r="W42" s="41"/>
-      <c r="X42" s="41"/>
-      <c r="Y42" s="41"/>
-      <c r="Z42" s="41"/>
-      <c r="AA42" s="41"/>
-      <c r="AB42" s="41"/>
-      <c r="AC42" s="41"/>
-      <c r="AD42" s="41"/>
-      <c r="AE42" s="17"/>
-      <c r="AF42" s="41"/>
-      <c r="AG42" s="41"/>
-      <c r="AH42" s="41"/>
-      <c r="AI42" s="41"/>
-      <c r="AJ42" s="41"/>
-      <c r="AK42" s="41"/>
-      <c r="AL42" s="41"/>
-      <c r="AM42" s="41"/>
-      <c r="AN42" s="41"/>
-      <c r="AO42" s="41"/>
+      <c r="T42" s="41">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="U42" s="41">
+        <v>0.09</v>
+      </c>
+      <c r="V42" s="41">
+        <v>5.22</v>
+      </c>
+      <c r="W42" s="41">
+        <v>7.2809999999999997</v>
+      </c>
+      <c r="X42" s="41">
+        <v>40.6</v>
+      </c>
+      <c r="Y42" s="41">
+        <v>61.6</v>
+      </c>
+      <c r="Z42" s="41">
+        <v>2.74</v>
+      </c>
+      <c r="AA42" s="41">
+        <v>155</v>
+      </c>
+      <c r="AB42" s="41">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="AC42" s="41">
+        <v>35.6</v>
+      </c>
+      <c r="AD42" s="41">
+        <v>50.1</v>
+      </c>
+      <c r="AE42" s="17">
+        <v>7.24</v>
+      </c>
+      <c r="AF42" s="41">
+        <v>410</v>
+      </c>
+      <c r="AG42" s="41">
+        <v>51</v>
+      </c>
+      <c r="AH42" s="41">
+        <v>7.3120000000000003</v>
+      </c>
+      <c r="AI42" s="41">
+        <v>33.9</v>
+      </c>
+      <c r="AJ42" s="41">
+        <v>3.4</v>
+      </c>
+      <c r="AK42" s="41">
+        <v>1.7</v>
+      </c>
+      <c r="AL42" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM42" s="41">
+        <v>7.5</v>
+      </c>
+      <c r="AN42" s="41">
+        <v>3.1</v>
+      </c>
+      <c r="AO42" s="41">
+        <v>199.8</v>
+      </c>
       <c r="AP42" s="74"/>
       <c r="AQ42" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="AR42" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>0.16650000000000001</v>
       </c>
       <c r="AS42" s="42">
         <f t="shared" si="23"/>
-        <v>-6.1</v>
+        <v>1.4000000000000004</v>
       </c>
       <c r="AT42" s="42">
         <f t="shared" si="24"/>
-        <v>-1.7</v>
+        <v>1.4000000000000001</v>
       </c>
       <c r="AU42" s="42">
         <f t="shared" si="25"/>
@@ -10203,36 +10445,38 @@
       <c r="BA42" s="43">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BB42" s="11"/>
+      <c r="BB42" s="11">
+        <v>0.02</v>
+      </c>
       <c r="BC42" s="43"/>
       <c r="BD42" s="22"/>
       <c r="BE42" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.366632E-3</v>
       </c>
       <c r="BF42" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>1.9679500800000003</v>
       </c>
       <c r="BG42" s="43">
         <f t="shared" si="45"/>
-        <v>188</v>
-      </c>
-      <c r="BH42" s="44" t="str">
+        <v>199.8</v>
+      </c>
+      <c r="BH42" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI42" s="44" t="str">
+        <v>3.7537537537537538E-2</v>
+      </c>
+      <c r="BI42" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>3.7499999999999999E-2</v>
       </c>
       <c r="BJ42" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>239.76000000000002</v>
       </c>
       <c r="BK42" s="44">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>0.16650000000000001</v>
       </c>
       <c r="BL42" s="44" t="str">
         <f t="shared" si="12"/>
@@ -10244,7 +10488,7 @@
       </c>
       <c r="BN42" s="44">
         <f t="shared" si="32"/>
-        <v>1.41</v>
+        <v>1.353645</v>
       </c>
       <c r="BO42" s="44" t="str">
         <f t="shared" si="49"/>
@@ -10252,15 +10496,15 @@
       </c>
       <c r="BP42" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>432.46753246753252</v>
       </c>
       <c r="BQ42" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>0.16650000000000001</v>
       </c>
       <c r="BR42" s="24">
         <f t="shared" si="54"/>
-        <v>1.41</v>
+        <v>1.353645</v>
       </c>
     </row>
     <row r="43" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -10279,59 +10523,123 @@
       <c r="E43" s="40">
         <v>4</v>
       </c>
-      <c r="G43" s="35"/>
+      <c r="G43" s="35">
+        <v>45572.404861111114</v>
+      </c>
       <c r="H43" s="40">
         <v>2119.61</v>
       </c>
       <c r="I43" s="41"/>
-      <c r="J43" s="41"/>
-      <c r="K43" s="41"/>
-      <c r="L43" s="41"/>
-      <c r="M43" s="41"/>
-      <c r="N43" s="41"/>
-      <c r="O43" s="41"/>
-      <c r="P43" s="41"/>
-      <c r="Q43" s="41"/>
-      <c r="R43" s="41"/>
+      <c r="J43" s="41">
+        <v>1739.34</v>
+      </c>
+      <c r="K43" s="41">
+        <v>25.9</v>
+      </c>
+      <c r="L43" s="41">
+        <v>23.9</v>
+      </c>
+      <c r="M43" s="41">
+        <v>92.1</v>
+      </c>
+      <c r="N43" s="41">
+        <v>16.7</v>
+      </c>
+      <c r="O43" s="41">
+        <v>333</v>
+      </c>
+      <c r="P43" s="41">
+        <v>1.4</v>
+      </c>
+      <c r="Q43" s="41">
+        <v>0.44</v>
+      </c>
+      <c r="R43" s="41">
+        <v>2.78</v>
+      </c>
       <c r="S43" s="41"/>
-      <c r="T43" s="41"/>
-      <c r="U43" s="41"/>
-      <c r="V43" s="41"/>
-      <c r="W43" s="41"/>
-      <c r="X43" s="41"/>
-      <c r="Y43" s="41"/>
-      <c r="Z43" s="41"/>
-      <c r="AA43" s="41"/>
-      <c r="AB43" s="41"/>
-      <c r="AC43" s="41"/>
-      <c r="AD43" s="41"/>
-      <c r="AE43" s="17"/>
-      <c r="AF43" s="41"/>
-      <c r="AG43" s="41"/>
-      <c r="AH43" s="41"/>
-      <c r="AI43" s="41"/>
-      <c r="AJ43" s="41"/>
-      <c r="AK43" s="41"/>
-      <c r="AL43" s="41"/>
-      <c r="AM43" s="41"/>
-      <c r="AN43" s="41"/>
-      <c r="AO43" s="41"/>
+      <c r="T43" s="41">
+        <v>0.17</v>
+      </c>
+      <c r="U43" s="41">
+        <v>0.08</v>
+      </c>
+      <c r="V43" s="41">
+        <v>3.71</v>
+      </c>
+      <c r="W43" s="41">
+        <v>7.2320000000000002</v>
+      </c>
+      <c r="X43" s="41">
+        <v>36.1</v>
+      </c>
+      <c r="Y43" s="41">
+        <v>56.8</v>
+      </c>
+      <c r="Z43" s="41">
+        <v>2.13</v>
+      </c>
+      <c r="AA43" s="41">
+        <v>138.1</v>
+      </c>
+      <c r="AB43" s="41">
+        <v>13.5</v>
+      </c>
+      <c r="AC43" s="41">
+        <v>31.7</v>
+      </c>
+      <c r="AD43" s="41">
+        <v>46.1</v>
+      </c>
+      <c r="AE43" s="17">
+        <v>7.1920000000000002</v>
+      </c>
+      <c r="AF43" s="41">
+        <v>412</v>
+      </c>
+      <c r="AG43" s="41">
+        <v>50.2</v>
+      </c>
+      <c r="AH43" s="41">
+        <v>7.2770000000000001</v>
+      </c>
+      <c r="AI43" s="41">
+        <v>33.9</v>
+      </c>
+      <c r="AJ43" s="41">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AK43" s="41">
+        <v>1.3</v>
+      </c>
+      <c r="AL43" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM43" s="41">
+        <v>7.6</v>
+      </c>
+      <c r="AN43" s="41">
+        <v>3.9</v>
+      </c>
+      <c r="AO43" s="41">
+        <v>199.2</v>
+      </c>
       <c r="AP43" s="74"/>
       <c r="AQ43" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.502</v>
       </c>
       <c r="AR43" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>0.16600000000000001</v>
       </c>
       <c r="AS43" s="42">
         <f t="shared" si="23"/>
-        <v>-4</v>
+        <v>3.5999999999999996</v>
       </c>
       <c r="AT43" s="42">
         <f t="shared" si="24"/>
-        <v>-2.5</v>
+        <v>1.4</v>
       </c>
       <c r="AU43" s="42">
         <f t="shared" si="25"/>
@@ -10355,35 +10663,37 @@
       <c r="BA43" s="43">
         <v>2.9999999999999997E-4</v>
       </c>
-      <c r="BB43" s="11"/>
+      <c r="BB43" s="11">
+        <v>0.02</v>
+      </c>
       <c r="BD43" s="22"/>
       <c r="BE43" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.4282639999999998E-3</v>
       </c>
       <c r="BF43" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.0567001599999997</v>
       </c>
       <c r="BG43" s="43">
         <f t="shared" si="45"/>
-        <v>188</v>
-      </c>
-      <c r="BH43" s="44" t="str">
+        <v>199.2</v>
+      </c>
+      <c r="BH43" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI43" s="44" t="str">
+        <v>3.8152610441767071E-2</v>
+      </c>
+      <c r="BI43" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>3.7999999999999999E-2</v>
       </c>
       <c r="BJ43" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>239.04</v>
       </c>
       <c r="BK43" s="44">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>0.16600000000000001</v>
       </c>
       <c r="BL43" s="45" t="str">
         <f t="shared" si="12"/>
@@ -10395,7 +10705,7 @@
       </c>
       <c r="BN43" s="44">
         <f t="shared" si="32"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
       <c r="BO43" s="44" t="str">
         <f t="shared" si="49"/>
@@ -10403,15 +10713,15 @@
       </c>
       <c r="BP43" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>431.16883116883122</v>
       </c>
       <c r="BQ43" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>0.16600000000000001</v>
       </c>
       <c r="BR43" s="24">
         <f t="shared" si="54"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -10430,59 +10740,123 @@
       <c r="E44" s="40">
         <v>4</v>
       </c>
-      <c r="G44" s="35"/>
+      <c r="G44" s="35">
+        <v>45572.40625</v>
+      </c>
       <c r="H44" s="40">
         <v>2119.61</v>
       </c>
       <c r="I44" s="41"/>
-      <c r="J44" s="41"/>
-      <c r="K44" s="41"/>
-      <c r="L44" s="41"/>
-      <c r="M44" s="41"/>
-      <c r="N44" s="41"/>
-      <c r="O44" s="41"/>
-      <c r="P44" s="41"/>
-      <c r="Q44" s="41"/>
-      <c r="R44" s="41"/>
+      <c r="J44" s="41">
+        <v>1851.24</v>
+      </c>
+      <c r="K44" s="41">
+        <v>26.4</v>
+      </c>
+      <c r="L44" s="41">
+        <v>24.8</v>
+      </c>
+      <c r="M44" s="41">
+        <v>94</v>
+      </c>
+      <c r="N44" s="41">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="O44" s="41">
+        <v>324</v>
+      </c>
+      <c r="P44" s="41">
+        <v>1.34</v>
+      </c>
+      <c r="Q44" s="41">
+        <v>0.39</v>
+      </c>
+      <c r="R44" s="41">
+        <v>1.64</v>
+      </c>
       <c r="S44" s="41"/>
-      <c r="T44" s="41"/>
-      <c r="U44" s="41"/>
-      <c r="V44" s="41"/>
-      <c r="W44" s="41"/>
-      <c r="X44" s="41"/>
-      <c r="Y44" s="41"/>
-      <c r="Z44" s="41"/>
-      <c r="AA44" s="41"/>
-      <c r="AB44" s="41"/>
-      <c r="AC44" s="41"/>
-      <c r="AD44" s="41"/>
-      <c r="AE44" s="17"/>
-      <c r="AF44" s="41"/>
-      <c r="AG44" s="41"/>
-      <c r="AH44" s="41"/>
-      <c r="AI44" s="41"/>
-      <c r="AJ44" s="41"/>
-      <c r="AK44" s="41"/>
-      <c r="AL44" s="41"/>
-      <c r="AM44" s="41"/>
-      <c r="AN44" s="41"/>
-      <c r="AO44" s="41"/>
+      <c r="T44" s="41">
+        <v>0.16</v>
+      </c>
+      <c r="U44" s="41">
+        <v>0.08</v>
+      </c>
+      <c r="V44" s="41">
+        <v>3.51</v>
+      </c>
+      <c r="W44" s="41">
+        <v>7.2720000000000002</v>
+      </c>
+      <c r="X44" s="41">
+        <v>32.4</v>
+      </c>
+      <c r="Y44" s="41">
+        <v>48.5</v>
+      </c>
+      <c r="Z44" s="41">
+        <v>2.2400000000000002</v>
+      </c>
+      <c r="AA44" s="41">
+        <v>139.4</v>
+      </c>
+      <c r="AB44" s="41">
+        <v>13.2</v>
+      </c>
+      <c r="AC44" s="41">
+        <v>28.5</v>
+      </c>
+      <c r="AD44" s="41">
+        <v>39.299999999999997</v>
+      </c>
+      <c r="AE44" s="17">
+        <v>7.2309999999999999</v>
+      </c>
+      <c r="AF44" s="41">
+        <v>407</v>
+      </c>
+      <c r="AG44" s="41">
+        <v>51</v>
+      </c>
+      <c r="AH44" s="41">
+        <v>7.298</v>
+      </c>
+      <c r="AI44" s="41">
+        <v>33.9</v>
+      </c>
+      <c r="AJ44" s="41">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AK44" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="AL44" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM44" s="41">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="AN44" s="41">
+        <v>3.6</v>
+      </c>
+      <c r="AO44" s="41">
+        <v>198.1</v>
+      </c>
       <c r="AP44" s="74"/>
       <c r="AQ44" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="AR44" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>0.14890513359397919</v>
       </c>
       <c r="AS44" s="42">
         <f t="shared" ref="AS44:AS75" si="55">AM44-AM35</f>
-        <v>-5.8</v>
+        <v>2.8999999999999995</v>
       </c>
       <c r="AT44" s="42">
         <f t="shared" ref="AT44:AT75" si="56">AN44-AN35</f>
-        <v>-2.6</v>
+        <v>1</v>
       </c>
       <c r="AU44" s="42">
         <f t="shared" ref="AU44:AU75" si="57">AP35-AP44</f>
@@ -10507,30 +10881,37 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BB44" s="11"/>
-      <c r="BD44" s="22"/>
+      <c r="BC44" s="81">
+        <f>0.00248175222656632*24*60/BG44</f>
+        <v>1.8039995993213025E-2</v>
+      </c>
+      <c r="BD44" s="81">
+        <f>0.176367129335544/BG44</f>
+        <v>8.9029343430360426E-4</v>
+      </c>
       <c r="BE44" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.4738639999999999E-3</v>
       </c>
       <c r="BF44" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.1223641599999996</v>
       </c>
       <c r="BG44" s="43">
         <f t="shared" si="45"/>
-        <v>188</v>
-      </c>
-      <c r="BH44" s="44" t="str">
+        <v>198.1</v>
+      </c>
+      <c r="BH44" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI44" s="44" t="str">
+        <v>4.3917213528520946E-2</v>
+      </c>
+      <c r="BI44" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>4.3499999999999997E-2</v>
       </c>
       <c r="BJ44" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>214.42339237533005</v>
       </c>
       <c r="BK44" s="44" t="str">
         <f t="shared" si="19"/>
@@ -10538,7 +10919,7 @@
       </c>
       <c r="BL44" s="45">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.14890513359397919</v>
       </c>
       <c r="BM44" s="45" t="str">
         <f t="shared" si="13"/>
@@ -10550,19 +10931,19 @@
       </c>
       <c r="BO44" s="44">
         <f t="shared" si="49"/>
-        <v>0</v>
+        <v>0.17636712933554399</v>
       </c>
       <c r="BP44" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>386.76658076358234</v>
       </c>
       <c r="BQ44" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>0.14890513359397919</v>
       </c>
       <c r="BR44" s="24">
         <f t="shared" si="54"/>
-        <v>0</v>
+        <v>0.17636712933554399</v>
       </c>
     </row>
     <row r="45" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -10581,59 +10962,123 @@
       <c r="E45" s="40">
         <v>4</v>
       </c>
-      <c r="G45" s="35"/>
+      <c r="G45" s="35">
+        <v>45572.406944444447</v>
+      </c>
       <c r="H45" s="40">
         <v>2119.61</v>
       </c>
       <c r="I45" s="41"/>
-      <c r="J45" s="41"/>
-      <c r="K45" s="41"/>
-      <c r="L45" s="41"/>
-      <c r="M45" s="41"/>
-      <c r="N45" s="41"/>
-      <c r="O45" s="41"/>
-      <c r="P45" s="41"/>
-      <c r="Q45" s="41"/>
-      <c r="R45" s="41"/>
+      <c r="J45" s="41">
+        <v>1865.34</v>
+      </c>
+      <c r="K45" s="41">
+        <v>28.1</v>
+      </c>
+      <c r="L45" s="41">
+        <v>26.4</v>
+      </c>
+      <c r="M45" s="41">
+        <v>94</v>
+      </c>
+      <c r="N45" s="41">
+        <v>16.7</v>
+      </c>
+      <c r="O45" s="41">
+        <v>325</v>
+      </c>
+      <c r="P45" s="41">
+        <v>1.4</v>
+      </c>
+      <c r="Q45" s="41">
+        <v>0.39</v>
+      </c>
+      <c r="R45" s="41">
+        <v>1.78</v>
+      </c>
       <c r="S45" s="41"/>
-      <c r="T45" s="41"/>
-      <c r="U45" s="41"/>
-      <c r="V45" s="41"/>
-      <c r="W45" s="41"/>
-      <c r="X45" s="41"/>
-      <c r="Y45" s="41"/>
-      <c r="Z45" s="41"/>
-      <c r="AA45" s="41"/>
-      <c r="AB45" s="41"/>
-      <c r="AC45" s="41"/>
-      <c r="AD45" s="41"/>
-      <c r="AE45" s="17"/>
-      <c r="AF45" s="41"/>
-      <c r="AG45" s="41"/>
-      <c r="AH45" s="41"/>
-      <c r="AI45" s="41"/>
-      <c r="AJ45" s="41"/>
-      <c r="AK45" s="41"/>
-      <c r="AL45" s="41"/>
-      <c r="AM45" s="41"/>
-      <c r="AN45" s="41"/>
-      <c r="AO45" s="41"/>
+      <c r="T45" s="41">
+        <v>0.16</v>
+      </c>
+      <c r="U45" s="41">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V45" s="41">
+        <v>3.47</v>
+      </c>
+      <c r="W45" s="41">
+        <v>7.26</v>
+      </c>
+      <c r="X45" s="41">
+        <v>33.1</v>
+      </c>
+      <c r="Y45" s="41">
+        <v>52.9</v>
+      </c>
+      <c r="Z45" s="41">
+        <v>2.17</v>
+      </c>
+      <c r="AA45" s="41">
+        <v>138</v>
+      </c>
+      <c r="AB45" s="41">
+        <v>13.2</v>
+      </c>
+      <c r="AC45" s="41">
+        <v>29.1</v>
+      </c>
+      <c r="AD45" s="41">
+        <v>43</v>
+      </c>
+      <c r="AE45" s="17">
+        <v>7.22</v>
+      </c>
+      <c r="AF45" s="41">
+        <v>409</v>
+      </c>
+      <c r="AG45" s="41">
+        <v>52.6</v>
+      </c>
+      <c r="AH45" s="41">
+        <v>7.3040000000000003</v>
+      </c>
+      <c r="AI45" s="41">
+        <v>33.9</v>
+      </c>
+      <c r="AJ45" s="41">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AK45" s="41">
+        <v>1</v>
+      </c>
+      <c r="AL45" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM45" s="41">
+        <v>8.5</v>
+      </c>
+      <c r="AN45" s="41">
+        <v>3.7</v>
+      </c>
+      <c r="AO45" s="41">
+        <v>198.9</v>
+      </c>
       <c r="AP45" s="74"/>
       <c r="AQ45" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.52600000000000002</v>
       </c>
       <c r="AR45" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>0.16320476690989325</v>
       </c>
       <c r="AS45" s="42">
         <f t="shared" si="55"/>
-        <v>-5.9</v>
+        <v>2.5999999999999996</v>
       </c>
       <c r="AT45" s="42">
         <f t="shared" si="56"/>
-        <v>-2.7</v>
+        <v>1</v>
       </c>
       <c r="AU45" s="42">
         <f t="shared" si="57"/>
@@ -10658,30 +11103,37 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="BB45" s="11"/>
-      <c r="BD45" s="22"/>
+      <c r="BC45" s="81">
+        <f>0.00272007944849822*24*60/BG45</f>
+        <v>1.9692882885054989E-2</v>
+      </c>
+      <c r="BD45" s="81">
+        <f>0.507148200573381/BG45</f>
+        <v>2.5497647087651129E-3</v>
+      </c>
       <c r="BE45" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.5752879999999998E-3</v>
       </c>
       <c r="BF45" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.26841472</v>
       </c>
       <c r="BG45" s="43">
         <f t="shared" si="45"/>
-        <v>188</v>
-      </c>
-      <c r="BH45" s="44" t="str">
+        <v>198.9</v>
+      </c>
+      <c r="BH45" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI45" s="44" t="str">
+        <v>4.2735042735042736E-2</v>
+      </c>
+      <c r="BI45" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>4.2500000000000003E-2</v>
       </c>
       <c r="BJ45" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>235.01486435024626</v>
       </c>
       <c r="BK45" s="44" t="str">
         <f t="shared" si="19"/>
@@ -10689,7 +11141,7 @@
       </c>
       <c r="BL45" s="45">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.16320476690989325</v>
       </c>
       <c r="BM45" s="45" t="str">
         <f t="shared" si="13"/>
@@ -10701,19 +11153,19 @@
       </c>
       <c r="BO45" s="44">
         <f t="shared" si="49"/>
-        <v>0</v>
+        <v>0.50714820057338095</v>
       </c>
       <c r="BP45" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>423.90848548024223</v>
       </c>
       <c r="BQ45" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>0.16320476690989325</v>
       </c>
       <c r="BR45" s="24">
         <f t="shared" si="54"/>
-        <v>0</v>
+        <v>0.50714820057338095</v>
       </c>
     </row>
     <row r="46" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -10732,58 +11184,122 @@
       <c r="E46" s="40">
         <v>4</v>
       </c>
-      <c r="G46" s="35"/>
+      <c r="G46" s="35">
+        <v>45572.407638888886</v>
+      </c>
       <c r="H46" s="40">
         <v>2119.61</v>
       </c>
-      <c r="J46" s="41"/>
-      <c r="K46" s="41"/>
-      <c r="L46" s="41"/>
-      <c r="M46" s="41"/>
-      <c r="N46" s="41"/>
-      <c r="O46" s="41"/>
-      <c r="P46" s="41"/>
-      <c r="Q46" s="41"/>
-      <c r="R46" s="41"/>
+      <c r="J46" s="41">
+        <v>1668.4349999999999</v>
+      </c>
+      <c r="K46" s="41">
+        <v>25.5</v>
+      </c>
+      <c r="L46" s="41">
+        <v>23.5</v>
+      </c>
+      <c r="M46" s="41">
+        <v>92.4</v>
+      </c>
+      <c r="N46" s="41">
+        <v>16.3</v>
+      </c>
+      <c r="O46" s="41">
+        <v>330</v>
+      </c>
+      <c r="P46" s="41">
+        <v>1.47</v>
+      </c>
+      <c r="Q46" s="41">
+        <v>0.44</v>
+      </c>
+      <c r="R46" s="41">
+        <v>1.81</v>
+      </c>
       <c r="S46" s="41"/>
-      <c r="T46" s="41"/>
-      <c r="U46" s="41"/>
-      <c r="V46" s="41"/>
-      <c r="W46" s="41"/>
-      <c r="X46" s="41"/>
-      <c r="Y46" s="41"/>
-      <c r="Z46" s="41"/>
-      <c r="AA46" s="41"/>
-      <c r="AB46" s="41"/>
-      <c r="AC46" s="41"/>
-      <c r="AD46" s="41"/>
-      <c r="AE46" s="17"/>
-      <c r="AF46" s="41"/>
-      <c r="AG46" s="41"/>
-      <c r="AH46" s="41"/>
-      <c r="AI46" s="41"/>
-      <c r="AJ46" s="41"/>
-      <c r="AK46" s="41"/>
-      <c r="AL46" s="41"/>
-      <c r="AM46" s="41"/>
-      <c r="AN46" s="41"/>
-      <c r="AO46" s="41"/>
+      <c r="T46" s="41">
+        <v>0.13</v>
+      </c>
+      <c r="U46" s="41">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="V46" s="41">
+        <v>3.76</v>
+      </c>
+      <c r="W46" s="41">
+        <v>7.27</v>
+      </c>
+      <c r="X46" s="41">
+        <v>53.6</v>
+      </c>
+      <c r="Y46" s="41">
+        <v>59.9</v>
+      </c>
+      <c r="Z46" s="41">
+        <v>2.6</v>
+      </c>
+      <c r="AA46" s="41">
+        <v>143</v>
+      </c>
+      <c r="AB46" s="41">
+        <v>21.8</v>
+      </c>
+      <c r="AC46" s="41">
+        <v>47</v>
+      </c>
+      <c r="AD46" s="41">
+        <v>48.7</v>
+      </c>
+      <c r="AE46" s="17">
+        <v>7.2290000000000001</v>
+      </c>
+      <c r="AF46" s="41">
+        <v>680</v>
+      </c>
+      <c r="AG46" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="AH46" s="41">
+        <v>7.2930000000000001</v>
+      </c>
+      <c r="AI46" s="41">
+        <v>33.9</v>
+      </c>
+      <c r="AJ46" s="41">
+        <v>2.6</v>
+      </c>
+      <c r="AK46" s="41">
+        <v>1.2</v>
+      </c>
+      <c r="AL46" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM46" s="41">
+        <v>5.7</v>
+      </c>
+      <c r="AN46" s="41">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AO46" s="41">
+        <v>198.4</v>
+      </c>
       <c r="AP46" s="74"/>
       <c r="AQ46" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="AR46" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>8.3923199999999989E-2</v>
       </c>
       <c r="AS46" s="42">
         <f t="shared" si="55"/>
-        <v>-3.7</v>
+        <v>2</v>
       </c>
       <c r="AT46" s="42">
         <f t="shared" si="56"/>
-        <v>-3</v>
+        <v>1.4000000000000004</v>
       </c>
       <c r="AU46" s="42">
         <f t="shared" si="57"/>
@@ -10811,27 +11327,27 @@
       <c r="BD46" s="22"/>
       <c r="BE46" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.3987199999999998E-3</v>
       </c>
       <c r="BF46" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.0141567999999994</v>
       </c>
       <c r="BG46" s="43">
         <f t="shared" si="45"/>
-        <v>188</v>
-      </c>
-      <c r="BH46" s="44" t="str">
+        <v>198.4</v>
+      </c>
+      <c r="BH46" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI46" s="44" t="str">
+        <v>2.8729838709677418E-2</v>
+      </c>
+      <c r="BI46" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>2.8500000000000001E-2</v>
       </c>
       <c r="BJ46" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>120.849408</v>
       </c>
       <c r="BK46" s="44" t="str">
         <f t="shared" si="19"/>
@@ -10843,11 +11359,11 @@
       </c>
       <c r="BM46" s="45">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>8.3923199999999989E-2</v>
       </c>
       <c r="BN46" s="44">
         <f t="shared" si="32"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
       <c r="BO46" s="44" t="str">
         <f t="shared" si="49"/>
@@ -10855,15 +11371,15 @@
       </c>
       <c r="BP46" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>217.98233766233764</v>
       </c>
       <c r="BQ46" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>8.3923199999999989E-2</v>
       </c>
       <c r="BR46" s="24">
         <f t="shared" si="54"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:70" s="40" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -10882,58 +11398,122 @@
       <c r="E47" s="40">
         <v>4</v>
       </c>
-      <c r="G47" s="35"/>
+      <c r="G47" s="35">
+        <v>45572.408333333333</v>
+      </c>
       <c r="H47" s="40">
         <v>2119.61</v>
       </c>
-      <c r="J47" s="41"/>
-      <c r="K47" s="41"/>
-      <c r="L47" s="41"/>
-      <c r="M47" s="41"/>
-      <c r="N47" s="41"/>
-      <c r="O47" s="41"/>
-      <c r="P47" s="41"/>
-      <c r="Q47" s="41"/>
-      <c r="R47" s="41"/>
+      <c r="J47" s="41">
+        <v>1775.5350000000001</v>
+      </c>
+      <c r="K47" s="41">
+        <v>26.8</v>
+      </c>
+      <c r="L47" s="41">
+        <v>25.3</v>
+      </c>
+      <c r="M47" s="41">
+        <v>94.3</v>
+      </c>
+      <c r="N47" s="41">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="O47" s="41">
+        <v>322</v>
+      </c>
+      <c r="P47" s="41">
+        <v>1.43</v>
+      </c>
+      <c r="Q47" s="41">
+        <v>0.41</v>
+      </c>
+      <c r="R47" s="41">
+        <v>2.1</v>
+      </c>
       <c r="S47" s="41"/>
-      <c r="T47" s="41"/>
-      <c r="U47" s="41"/>
-      <c r="V47" s="41"/>
-      <c r="W47" s="41"/>
-      <c r="X47" s="41"/>
-      <c r="Y47" s="41"/>
-      <c r="Z47" s="41"/>
-      <c r="AA47" s="41"/>
-      <c r="AB47" s="41"/>
-      <c r="AC47" s="41"/>
-      <c r="AD47" s="41"/>
-      <c r="AE47" s="17"/>
-      <c r="AF47" s="41"/>
-      <c r="AG47" s="41"/>
-      <c r="AH47" s="41"/>
-      <c r="AI47" s="41"/>
-      <c r="AJ47" s="41"/>
-      <c r="AK47" s="41"/>
-      <c r="AL47" s="41"/>
-      <c r="AM47" s="41"/>
-      <c r="AN47" s="41"/>
-      <c r="AO47" s="41"/>
+      <c r="T47" s="41">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="U47" s="41">
+        <v>0.08</v>
+      </c>
+      <c r="V47" s="41">
+        <v>3.38</v>
+      </c>
+      <c r="W47" s="41">
+        <v>7.2690000000000001</v>
+      </c>
+      <c r="X47" s="41">
+        <v>43.2</v>
+      </c>
+      <c r="Y47" s="41">
+        <v>60.6</v>
+      </c>
+      <c r="Z47" s="41">
+        <v>2.66</v>
+      </c>
+      <c r="AA47" s="41">
+        <v>137.4</v>
+      </c>
+      <c r="AB47" s="41">
+        <v>17.5</v>
+      </c>
+      <c r="AC47" s="41">
+        <v>37.9</v>
+      </c>
+      <c r="AD47" s="41">
+        <v>49.3</v>
+      </c>
+      <c r="AE47" s="17">
+        <v>7.2290000000000001</v>
+      </c>
+      <c r="AF47" s="41">
+        <v>469</v>
+      </c>
+      <c r="AG47" s="41">
+        <v>22.8</v>
+      </c>
+      <c r="AH47" s="41">
+        <v>7.298</v>
+      </c>
+      <c r="AI47" s="41">
+        <v>33.9</v>
+      </c>
+      <c r="AJ47" s="41">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AK47" s="41">
+        <v>1.4</v>
+      </c>
+      <c r="AL47" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM47" s="41">
+        <v>5.9</v>
+      </c>
+      <c r="AN47" s="41">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AO47" s="41">
+        <v>198.2</v>
+      </c>
       <c r="AP47" s="75"/>
       <c r="AQ47" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.22800000000000001</v>
       </c>
       <c r="AR47" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>9.0260279999999998E-2</v>
       </c>
       <c r="AS47" s="42">
         <f t="shared" si="55"/>
-        <v>-3.9</v>
+        <v>2.0000000000000004</v>
       </c>
       <c r="AT47" s="42">
         <f t="shared" si="56"/>
-        <v>-3.1</v>
+        <v>1.3000000000000003</v>
       </c>
       <c r="AU47" s="42">
         <f t="shared" si="57"/>
@@ -10961,27 +11541,27 @@
       <c r="BD47" s="22"/>
       <c r="BE47" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.5043379999999998E-3</v>
       </c>
       <c r="BF47" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.1662467199999997</v>
       </c>
       <c r="BG47" s="43">
         <f t="shared" si="45"/>
-        <v>188</v>
-      </c>
-      <c r="BH47" s="44" t="str">
+        <v>198.2</v>
+      </c>
+      <c r="BH47" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI47" s="44" t="str">
+        <v>2.9767911200807268E-2</v>
+      </c>
+      <c r="BI47" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>2.9500000000000002E-2</v>
       </c>
       <c r="BJ47" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>129.9748032</v>
       </c>
       <c r="BK47" s="44" t="str">
         <f t="shared" si="19"/>
@@ -10993,11 +11573,11 @@
       </c>
       <c r="BM47" s="45">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>9.0260279999999998E-2</v>
       </c>
       <c r="BN47" s="44">
         <f t="shared" si="32"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
       <c r="BO47" s="44" t="str">
         <f t="shared" si="49"/>
@@ -11005,15 +11585,15 @@
       </c>
       <c r="BP47" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>234.44228571428573</v>
       </c>
       <c r="BQ47" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>9.0260279999999998E-2</v>
       </c>
       <c r="BR47" s="24">
         <f t="shared" si="54"/>
-        <v>1.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -11033,24 +11613,38 @@
         <v>5</v>
       </c>
       <c r="F48" s="3"/>
-      <c r="G48" s="34"/>
+      <c r="G48" s="34">
+        <v>45573.359722222223</v>
+      </c>
       <c r="H48" s="3">
         <v>2716.05</v>
       </c>
       <c r="I48" s="3"/>
-      <c r="J48" s="6"/>
-      <c r="K48" s="6"/>
-      <c r="L48" s="6"/>
-      <c r="M48" s="6"/>
+      <c r="J48" s="6">
+        <v>1932.48</v>
+      </c>
+      <c r="K48" s="6">
+        <v>22.2</v>
+      </c>
+      <c r="L48" s="6">
+        <v>21.1</v>
+      </c>
+      <c r="M48" s="6">
+        <v>95</v>
+      </c>
       <c r="N48" s="6"/>
       <c r="O48" s="6"/>
       <c r="P48" s="6"/>
       <c r="Q48" s="6"/>
-      <c r="R48" s="6"/>
+      <c r="R48" s="6">
+        <v>2.31</v>
+      </c>
       <c r="S48" s="6"/>
       <c r="T48" s="6"/>
       <c r="U48" s="6"/>
-      <c r="V48" s="6"/>
+      <c r="V48" s="6">
+        <v>2.23</v>
+      </c>
       <c r="W48" s="6"/>
       <c r="X48" s="6"/>
       <c r="Y48" s="6"/>
@@ -11059,21 +11653,33 @@
       <c r="AB48" s="6"/>
       <c r="AC48" s="6"/>
       <c r="AD48" s="6"/>
-      <c r="AE48" s="16"/>
+      <c r="AE48" s="16">
+        <v>7.31</v>
+      </c>
       <c r="AF48" s="6"/>
-      <c r="AG48" s="6"/>
+      <c r="AG48" s="6">
+        <v>49.9998439730619</v>
+      </c>
       <c r="AH48" s="6"/>
-      <c r="AI48" s="6"/>
+      <c r="AI48" s="6">
+        <v>33.998356455407396</v>
+      </c>
       <c r="AJ48" s="6"/>
       <c r="AK48" s="6"/>
       <c r="AL48" s="6"/>
-      <c r="AM48" s="6"/>
-      <c r="AN48" s="6"/>
-      <c r="AO48" s="6"/>
+      <c r="AM48" s="6">
+        <v>35159.5078125</v>
+      </c>
+      <c r="AN48" s="6">
+        <v>17535.712890625</v>
+      </c>
+      <c r="AO48" s="6">
+        <v>617400</v>
+      </c>
       <c r="AP48" s="72"/>
       <c r="AQ48" s="32">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.49999843973061897</v>
       </c>
       <c r="AR48" s="32">
         <f t="shared" si="50"/>
@@ -11081,11 +11687,11 @@
       </c>
       <c r="AS48" s="32">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>12852.744140625</v>
       </c>
       <c r="AT48" s="32">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>2616.2060546875</v>
       </c>
       <c r="AU48" s="32">
         <f t="shared" si="57"/>
@@ -11111,26 +11717,29 @@
       </c>
       <c r="BB48" s="8"/>
       <c r="BC48" s="9"/>
-      <c r="BD48" s="21"/>
+      <c r="BD48" s="21">
+        <f>3886.90413432793/BG48</f>
+        <v>6.2956011245998223E-3</v>
+      </c>
       <c r="BE48" s="9">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>5.2108560000000006</v>
       </c>
       <c r="BF48" s="9">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>7503.6326400000016</v>
       </c>
       <c r="BG48" s="9">
         <f t="shared" si="45"/>
-        <v>591640</v>
-      </c>
-      <c r="BH48" s="10" t="str">
+        <v>617400</v>
+      </c>
+      <c r="BH48" s="10">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI48" s="10" t="str">
+        <v>5.6947696489310008E-2</v>
+      </c>
+      <c r="BI48" s="10">
         <f t="shared" si="47"/>
-        <v/>
+        <v>5.9391060494087836E-2</v>
       </c>
       <c r="BJ48" s="10">
         <f t="shared" si="48"/>
@@ -11154,7 +11763,7 @@
       </c>
       <c r="BO48" s="10">
         <f t="shared" si="49"/>
-        <v>0</v>
+        <v>3886.9041343279305</v>
       </c>
       <c r="BP48" s="62">
         <f t="shared" si="52"/>
@@ -11166,7 +11775,7 @@
       </c>
       <c r="BR48" s="26">
         <f t="shared" si="54"/>
-        <v>0</v>
+        <v>3886.9041343279305</v>
       </c>
     </row>
     <row r="49" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -11185,54 +11794,118 @@
       <c r="E49" s="40">
         <v>5</v>
       </c>
-      <c r="G49" s="35"/>
+      <c r="G49" s="35">
+        <v>45573.445590277777</v>
+      </c>
       <c r="H49" s="40">
         <v>2716.05</v>
       </c>
-      <c r="J49" s="41"/>
-      <c r="K49" s="41"/>
-      <c r="L49" s="41"/>
-      <c r="M49" s="41"/>
-      <c r="N49" s="41"/>
-      <c r="O49" s="41"/>
-      <c r="P49" s="41"/>
-      <c r="Q49" s="41"/>
-      <c r="R49" s="41"/>
+      <c r="J49" s="41">
+        <v>2466.585</v>
+      </c>
+      <c r="K49" s="41">
+        <v>23.280999999999999</v>
+      </c>
+      <c r="L49" s="41">
+        <v>21.760999999999999</v>
+      </c>
+      <c r="M49" s="41">
+        <v>93.5</v>
+      </c>
+      <c r="N49" s="41">
+        <v>15.73</v>
+      </c>
+      <c r="O49" s="41">
+        <v>322</v>
+      </c>
+      <c r="P49" s="41">
+        <v>1.43</v>
+      </c>
+      <c r="Q49" s="41">
+        <v>0.37</v>
+      </c>
+      <c r="R49" s="41">
+        <v>2.25</v>
+      </c>
       <c r="S49" s="41"/>
-      <c r="T49" s="41"/>
-      <c r="U49" s="41"/>
-      <c r="V49" s="41"/>
-      <c r="W49" s="41"/>
-      <c r="X49" s="41"/>
-      <c r="Y49" s="41"/>
-      <c r="Z49" s="41"/>
-      <c r="AA49" s="41"/>
-      <c r="AB49" s="41"/>
-      <c r="AC49" s="41"/>
-      <c r="AD49" s="41"/>
-      <c r="AE49" s="17"/>
-      <c r="AF49" s="41"/>
-      <c r="AG49" s="41"/>
-      <c r="AH49" s="41"/>
-      <c r="AI49" s="41"/>
-      <c r="AJ49" s="41"/>
-      <c r="AK49" s="41"/>
-      <c r="AL49" s="41"/>
-      <c r="AM49" s="41"/>
-      <c r="AN49" s="41"/>
-      <c r="AO49" s="41"/>
+      <c r="T49" s="41">
+        <v>0.15</v>
+      </c>
+      <c r="U49" s="41">
+        <v>0.11</v>
+      </c>
+      <c r="V49" s="41">
+        <v>2.7</v>
+      </c>
+      <c r="W49" s="41">
+        <v>7.266</v>
+      </c>
+      <c r="X49" s="41">
+        <v>46.3</v>
+      </c>
+      <c r="Y49" s="41">
+        <v>66.3</v>
+      </c>
+      <c r="Z49" s="41">
+        <v>2.64</v>
+      </c>
+      <c r="AA49" s="41">
+        <v>136.4</v>
+      </c>
+      <c r="AB49" s="41">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="AC49" s="41">
+        <v>40.6</v>
+      </c>
+      <c r="AD49" s="41">
+        <v>54</v>
+      </c>
+      <c r="AE49" s="17">
+        <v>7.2249999999999996</v>
+      </c>
+      <c r="AF49" s="41">
+        <v>407</v>
+      </c>
+      <c r="AG49" s="41">
+        <v>50.8</v>
+      </c>
+      <c r="AH49" s="41">
+        <v>7.3070000000000004</v>
+      </c>
+      <c r="AI49" s="41">
+        <v>34</v>
+      </c>
+      <c r="AJ49" s="41">
+        <v>2</v>
+      </c>
+      <c r="AK49" s="41">
+        <v>2.9</v>
+      </c>
+      <c r="AL49" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM49" s="41">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="AN49" s="41">
+        <v>4</v>
+      </c>
+      <c r="AO49" s="41">
+        <v>197</v>
+      </c>
       <c r="AP49" s="74"/>
       <c r="AQ49" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.50800000000000001</v>
       </c>
       <c r="AR49" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>0.10288600799999999</v>
       </c>
       <c r="AS49" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>2.2000000000000011</v>
       </c>
       <c r="AT49" s="42">
         <f t="shared" si="56"/>
@@ -11265,27 +11938,27 @@
       <c r="BD49" s="22"/>
       <c r="BE49" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.7147667999999998E-3</v>
       </c>
       <c r="BF49" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.4692641919999998</v>
       </c>
       <c r="BG49" s="43">
         <f t="shared" si="45"/>
-        <v>185.6</v>
-      </c>
-      <c r="BH49" s="44" t="str">
+        <v>197</v>
+      </c>
+      <c r="BH49" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI49" s="44" t="str">
+        <v>4.2131979695431476E-2</v>
+      </c>
+      <c r="BI49" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>4.1500000000000002E-2</v>
       </c>
       <c r="BJ49" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>148.15585152</v>
       </c>
       <c r="BK49" s="44" t="str">
         <f t="shared" si="19"/>
@@ -11297,11 +11970,11 @@
       </c>
       <c r="BM49" s="45">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.10288600799999999</v>
       </c>
       <c r="BN49" s="44">
         <f t="shared" si="32"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
       <c r="BO49" s="44" t="str">
         <f t="shared" si="49"/>
@@ -11309,15 +11982,15 @@
       </c>
       <c r="BP49" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>267.23638441558438</v>
       </c>
       <c r="BQ49" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>0.10288600799999999</v>
       </c>
       <c r="BR49" s="24">
         <f t="shared" si="54"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -11336,54 +12009,118 @@
       <c r="E50" s="40">
         <v>5</v>
       </c>
-      <c r="G50" s="35"/>
+      <c r="G50" s="35">
+        <v>45573.421898148146</v>
+      </c>
       <c r="H50" s="40">
         <v>2716.05</v>
       </c>
-      <c r="J50" s="41"/>
-      <c r="K50" s="41"/>
-      <c r="L50" s="41"/>
-      <c r="M50" s="41"/>
-      <c r="N50" s="41"/>
-      <c r="O50" s="41"/>
-      <c r="P50" s="41"/>
-      <c r="Q50" s="41"/>
-      <c r="R50" s="41"/>
+      <c r="J50" s="41">
+        <v>2406.1950000000002</v>
+      </c>
+      <c r="K50" s="41">
+        <v>27.155999999999999</v>
+      </c>
+      <c r="L50" s="41">
+        <v>25.081</v>
+      </c>
+      <c r="M50" s="41">
+        <v>92.4</v>
+      </c>
+      <c r="N50" s="41">
+        <v>15.18</v>
+      </c>
+      <c r="O50" s="41">
+        <v>325</v>
+      </c>
+      <c r="P50" s="41">
+        <v>1.38</v>
+      </c>
+      <c r="Q50" s="41">
+        <v>0.37</v>
+      </c>
+      <c r="R50" s="41">
+        <v>2.25</v>
+      </c>
       <c r="S50" s="41"/>
-      <c r="T50" s="41"/>
-      <c r="U50" s="41"/>
-      <c r="V50" s="41"/>
-      <c r="W50" s="41"/>
-      <c r="X50" s="41"/>
-      <c r="Y50" s="41"/>
-      <c r="Z50" s="41"/>
-      <c r="AA50" s="41"/>
-      <c r="AB50" s="41"/>
-      <c r="AC50" s="41"/>
-      <c r="AD50" s="41"/>
-      <c r="AE50" s="17"/>
-      <c r="AF50" s="41"/>
-      <c r="AG50" s="41"/>
-      <c r="AH50" s="41"/>
-      <c r="AI50" s="41"/>
-      <c r="AJ50" s="41"/>
-      <c r="AK50" s="41"/>
-      <c r="AL50" s="41"/>
-      <c r="AM50" s="41"/>
-      <c r="AN50" s="41"/>
-      <c r="AO50" s="41"/>
+      <c r="T50" s="41">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="U50" s="41">
+        <v>0.11</v>
+      </c>
+      <c r="V50" s="41">
+        <v>3.08</v>
+      </c>
+      <c r="W50" s="41">
+        <v>7.2430000000000003</v>
+      </c>
+      <c r="X50" s="41">
+        <v>33.799999999999997</v>
+      </c>
+      <c r="Y50" s="41">
+        <v>66</v>
+      </c>
+      <c r="Z50" s="41">
+        <v>2.75</v>
+      </c>
+      <c r="AA50" s="41">
+        <v>136.19999999999999</v>
+      </c>
+      <c r="AB50" s="41">
+        <v>12.9</v>
+      </c>
+      <c r="AC50" s="41">
+        <v>29.6</v>
+      </c>
+      <c r="AD50" s="41">
+        <v>53.8</v>
+      </c>
+      <c r="AE50" s="17">
+        <v>7.2030000000000003</v>
+      </c>
+      <c r="AF50" s="41">
+        <v>408</v>
+      </c>
+      <c r="AG50" s="41">
+        <v>49.9</v>
+      </c>
+      <c r="AH50" s="41">
+        <v>7.2830000000000004</v>
+      </c>
+      <c r="AI50" s="41">
+        <v>34</v>
+      </c>
+      <c r="AJ50" s="41">
+        <v>2.1</v>
+      </c>
+      <c r="AK50" s="41">
+        <v>2.8</v>
+      </c>
+      <c r="AL50" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM50" s="41">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="AN50" s="41">
+        <v>4.3</v>
+      </c>
+      <c r="AO50" s="41">
+        <v>197.6</v>
+      </c>
       <c r="AP50" s="74"/>
       <c r="AQ50" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.499</v>
       </c>
       <c r="AR50" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>0.11894413440000001</v>
       </c>
       <c r="AS50" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>2.1999999999999993</v>
       </c>
       <c r="AT50" s="42">
         <f t="shared" si="56"/>
@@ -11416,27 +12153,27 @@
       <c r="BD50" s="22"/>
       <c r="BE50" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.9824022400000002E-3</v>
       </c>
       <c r="BF50" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.8546592256000003</v>
       </c>
       <c r="BG50" s="43">
         <f t="shared" si="45"/>
-        <v>185.6</v>
-      </c>
-      <c r="BH50" s="44" t="str">
+        <v>197.6</v>
+      </c>
+      <c r="BH50" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI50" s="44" t="str">
+        <v>4.149797570850202E-2</v>
+      </c>
+      <c r="BI50" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>4.0999999999999995E-2</v>
       </c>
       <c r="BJ50" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>171.27955353600001</v>
       </c>
       <c r="BK50" s="44" t="str">
         <f t="shared" si="19"/>
@@ -11448,11 +12185,11 @@
       </c>
       <c r="BM50" s="45">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>0.11894413440000001</v>
       </c>
       <c r="BN50" s="44">
         <f t="shared" si="32"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
       <c r="BO50" s="44" t="str">
         <f t="shared" si="49"/>
@@ -11460,15 +12197,15 @@
       </c>
       <c r="BP50" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>308.94580363636368</v>
       </c>
       <c r="BQ50" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>0.11894413440000001</v>
       </c>
       <c r="BR50" s="24">
         <f t="shared" si="54"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -11487,46 +12224,110 @@
       <c r="E51" s="40">
         <v>5</v>
       </c>
-      <c r="G51" s="35"/>
+      <c r="G51" s="35">
+        <v>45573.422743055555</v>
+      </c>
       <c r="H51" s="40">
         <v>2716.05</v>
       </c>
-      <c r="J51" s="41"/>
-      <c r="K51" s="41"/>
-      <c r="L51" s="41"/>
-      <c r="M51" s="41"/>
-      <c r="N51" s="41"/>
-      <c r="O51" s="41"/>
-      <c r="P51" s="41"/>
-      <c r="Q51" s="41"/>
-      <c r="R51" s="41"/>
+      <c r="J51" s="41">
+        <v>2279.1149999999998</v>
+      </c>
+      <c r="K51" s="41">
+        <v>23.099</v>
+      </c>
+      <c r="L51" s="41">
+        <v>20.533000000000001</v>
+      </c>
+      <c r="M51" s="41">
+        <v>88.9</v>
+      </c>
+      <c r="N51" s="41">
+        <v>16.61</v>
+      </c>
+      <c r="O51" s="41">
+        <v>374</v>
+      </c>
+      <c r="P51" s="41">
+        <v>1.19</v>
+      </c>
+      <c r="Q51" s="41">
+        <v>0.39</v>
+      </c>
+      <c r="R51" s="41">
+        <v>3.27</v>
+      </c>
       <c r="S51" s="41"/>
-      <c r="T51" s="41"/>
-      <c r="U51" s="41"/>
-      <c r="V51" s="41"/>
-      <c r="W51" s="41"/>
-      <c r="X51" s="41"/>
-      <c r="Y51" s="41"/>
-      <c r="Z51" s="41"/>
-      <c r="AA51" s="41"/>
-      <c r="AB51" s="41"/>
-      <c r="AC51" s="41"/>
-      <c r="AD51" s="41"/>
-      <c r="AE51" s="17"/>
-      <c r="AF51" s="41"/>
-      <c r="AG51" s="41"/>
-      <c r="AH51" s="41"/>
-      <c r="AI51" s="41"/>
-      <c r="AJ51" s="41"/>
-      <c r="AK51" s="41"/>
-      <c r="AL51" s="41"/>
-      <c r="AM51" s="41"/>
-      <c r="AN51" s="41"/>
-      <c r="AO51" s="41"/>
+      <c r="T51" s="41">
+        <v>0.18</v>
+      </c>
+      <c r="U51" s="41">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="V51" s="41">
+        <v>4.45</v>
+      </c>
+      <c r="W51" s="41">
+        <v>7.2389999999999999</v>
+      </c>
+      <c r="X51" s="41">
+        <v>39.1</v>
+      </c>
+      <c r="Y51" s="41">
+        <v>52.2</v>
+      </c>
+      <c r="Z51" s="41">
+        <v>1.85</v>
+      </c>
+      <c r="AA51" s="41">
+        <v>153.9</v>
+      </c>
+      <c r="AB51" s="41">
+        <v>14.8</v>
+      </c>
+      <c r="AC51" s="41">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="AD51" s="41">
+        <v>42.4</v>
+      </c>
+      <c r="AE51" s="17">
+        <v>7.1989999999999998</v>
+      </c>
+      <c r="AF51" s="41">
+        <v>407</v>
+      </c>
+      <c r="AG51" s="41">
+        <v>49.1</v>
+      </c>
+      <c r="AH51" s="41">
+        <v>7.2430000000000003</v>
+      </c>
+      <c r="AI51" s="41">
+        <v>34</v>
+      </c>
+      <c r="AJ51" s="41">
+        <v>3.4</v>
+      </c>
+      <c r="AK51" s="41">
+        <v>2.7</v>
+      </c>
+      <c r="AL51" s="41">
+        <v>0.2</v>
+      </c>
+      <c r="AM51" s="41">
+        <v>11.3</v>
+      </c>
+      <c r="AN51" s="41">
+        <v>4.5</v>
+      </c>
+      <c r="AO51" s="41">
+        <v>202.2</v>
+      </c>
       <c r="AP51" s="74"/>
       <c r="AQ51" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.49099999999999999</v>
       </c>
       <c r="AR51" s="42">
         <f t="shared" si="50"/>
@@ -11534,11 +12335,11 @@
       </c>
       <c r="AS51" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>3.8000000000000007</v>
       </c>
       <c r="AT51" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="AU51" s="42">
         <f t="shared" si="57"/>
@@ -11567,23 +12368,23 @@
       <c r="BD51" s="22"/>
       <c r="BE51" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.6607090400000001E-3</v>
       </c>
       <c r="BF51" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.3914210176000004</v>
       </c>
       <c r="BG51" s="43">
         <f t="shared" si="45"/>
-        <v>185.6</v>
-      </c>
-      <c r="BH51" s="44" t="str">
+        <v>202.2</v>
+      </c>
+      <c r="BH51" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI51" s="44" t="str">
+        <v>5.5885262116716128E-2</v>
+      </c>
+      <c r="BI51" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>5.6500000000000002E-2</v>
       </c>
       <c r="BJ51" s="44">
         <f t="shared" si="48"/>
@@ -11603,7 +12404,7 @@
       </c>
       <c r="BN51" s="44">
         <f t="shared" si="32"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
       <c r="BO51" s="44" t="str">
         <f t="shared" si="49"/>
@@ -11619,7 +12420,7 @@
       </c>
       <c r="BR51" s="24">
         <f t="shared" si="54"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -11638,46 +12439,110 @@
       <c r="E52" s="40">
         <v>5</v>
       </c>
-      <c r="G52" s="35"/>
+      <c r="G52" s="35">
+        <v>45573.423587962963</v>
+      </c>
       <c r="H52" s="40">
         <v>2716.05</v>
       </c>
-      <c r="J52" s="41"/>
-      <c r="K52" s="41"/>
-      <c r="L52" s="41"/>
-      <c r="M52" s="41"/>
-      <c r="N52" s="41"/>
-      <c r="O52" s="41"/>
-      <c r="P52" s="41"/>
-      <c r="Q52" s="41"/>
-      <c r="R52" s="41"/>
+      <c r="J52" s="41">
+        <v>2461.2449999999999</v>
+      </c>
+      <c r="K52" s="41">
+        <v>21.51</v>
+      </c>
+      <c r="L52" s="41">
+        <v>19.835999999999999</v>
+      </c>
+      <c r="M52" s="41">
+        <v>92.2</v>
+      </c>
+      <c r="N52" s="41">
+        <v>16.559999999999999</v>
+      </c>
+      <c r="O52" s="41">
+        <v>339</v>
+      </c>
+      <c r="P52" s="41">
+        <v>1.26</v>
+      </c>
+      <c r="Q52" s="41">
+        <v>0.39</v>
+      </c>
+      <c r="R52" s="41">
+        <v>2.81</v>
+      </c>
       <c r="S52" s="41"/>
-      <c r="T52" s="41"/>
-      <c r="U52" s="41"/>
-      <c r="V52" s="41"/>
-      <c r="W52" s="41"/>
-      <c r="X52" s="41"/>
-      <c r="Y52" s="41"/>
-      <c r="Z52" s="41"/>
-      <c r="AA52" s="41"/>
-      <c r="AB52" s="41"/>
-      <c r="AC52" s="41"/>
-      <c r="AD52" s="41"/>
-      <c r="AE52" s="17"/>
-      <c r="AF52" s="41"/>
-      <c r="AG52" s="41"/>
-      <c r="AH52" s="41"/>
-      <c r="AI52" s="41"/>
-      <c r="AJ52" s="41"/>
-      <c r="AK52" s="41"/>
-      <c r="AL52" s="41"/>
-      <c r="AM52" s="41"/>
-      <c r="AN52" s="41"/>
-      <c r="AO52" s="41"/>
+      <c r="T52" s="41">
+        <v>0.2</v>
+      </c>
+      <c r="U52" s="41">
+        <v>0.12</v>
+      </c>
+      <c r="V52" s="41">
+        <v>3.34</v>
+      </c>
+      <c r="W52" s="41">
+        <v>7.2460000000000004</v>
+      </c>
+      <c r="X52" s="41">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="Y52" s="41">
+        <v>47.5</v>
+      </c>
+      <c r="Z52" s="41">
+        <v>1.82</v>
+      </c>
+      <c r="AA52" s="41">
+        <v>143.19999999999999</v>
+      </c>
+      <c r="AB52" s="41">
+        <v>13.7</v>
+      </c>
+      <c r="AC52" s="41">
+        <v>31.3</v>
+      </c>
+      <c r="AD52" s="41">
+        <v>38.5</v>
+      </c>
+      <c r="AE52" s="17">
+        <v>7.2060000000000004</v>
+      </c>
+      <c r="AF52" s="41">
+        <v>409</v>
+      </c>
+      <c r="AG52" s="41">
+        <v>49.7</v>
+      </c>
+      <c r="AH52" s="41">
+        <v>7.2539999999999996</v>
+      </c>
+      <c r="AI52" s="41">
+        <v>34</v>
+      </c>
+      <c r="AJ52" s="41">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AK52" s="41">
+        <v>2</v>
+      </c>
+      <c r="AL52" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM52" s="41">
+        <v>11.7</v>
+      </c>
+      <c r="AN52" s="41">
+        <v>3.9</v>
+      </c>
+      <c r="AO52" s="41">
+        <v>200.1</v>
+      </c>
       <c r="AP52" s="74"/>
       <c r="AQ52" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.49700000000000005</v>
       </c>
       <c r="AR52" s="42">
         <f t="shared" si="50"/>
@@ -11685,7 +12550,7 @@
       </c>
       <c r="AS52" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="AT52" s="42">
         <f t="shared" si="56"/>
@@ -11717,23 +12582,23 @@
       <c r="BD52" s="22"/>
       <c r="BE52" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.5876734399999999E-3</v>
       </c>
       <c r="BF52" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.2862497535999999</v>
       </c>
       <c r="BG52" s="43">
         <f t="shared" si="45"/>
-        <v>185.6</v>
-      </c>
-      <c r="BH52" s="44" t="str">
+        <v>200.1</v>
+      </c>
+      <c r="BH52" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI52" s="44" t="str">
+        <v>5.847076461769115E-2</v>
+      </c>
+      <c r="BI52" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>5.8499999999999996E-2</v>
       </c>
       <c r="BJ52" s="44">
         <f t="shared" si="48"/>
@@ -11753,7 +12618,7 @@
       </c>
       <c r="BN52" s="44">
         <f t="shared" si="32"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
       <c r="BO52" s="44" t="str">
         <f t="shared" si="49"/>
@@ -11769,7 +12634,7 @@
       </c>
       <c r="BR52" s="24">
         <f t="shared" si="54"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -11788,46 +12653,110 @@
       <c r="E53" s="40">
         <v>5</v>
       </c>
-      <c r="G53" s="35"/>
+      <c r="G53" s="35">
+        <v>45573.424444444441</v>
+      </c>
       <c r="H53" s="40">
         <v>2716.05</v>
       </c>
-      <c r="J53" s="41"/>
-      <c r="K53" s="41"/>
-      <c r="L53" s="41"/>
-      <c r="M53" s="41"/>
-      <c r="N53" s="41"/>
-      <c r="O53" s="41"/>
-      <c r="P53" s="41"/>
-      <c r="Q53" s="41"/>
-      <c r="R53" s="41"/>
+      <c r="J53" s="41">
+        <v>2561.79</v>
+      </c>
+      <c r="K53" s="41">
+        <v>22.911999999999999</v>
+      </c>
+      <c r="L53" s="41">
+        <v>21.283000000000001</v>
+      </c>
+      <c r="M53" s="41">
+        <v>92.9</v>
+      </c>
+      <c r="N53" s="41">
+        <v>16.23</v>
+      </c>
+      <c r="O53" s="41">
+        <v>327</v>
+      </c>
+      <c r="P53" s="41">
+        <v>1.3</v>
+      </c>
+      <c r="Q53" s="41">
+        <v>0.35</v>
+      </c>
+      <c r="R53" s="41">
+        <v>1.49</v>
+      </c>
       <c r="S53" s="41"/>
-      <c r="T53" s="41"/>
-      <c r="U53" s="41"/>
-      <c r="V53" s="41"/>
-      <c r="W53" s="41"/>
-      <c r="X53" s="41"/>
-      <c r="Y53" s="41"/>
-      <c r="Z53" s="41"/>
-      <c r="AA53" s="41"/>
-      <c r="AB53" s="41"/>
-      <c r="AC53" s="41"/>
-      <c r="AD53" s="41"/>
-      <c r="AE53" s="17"/>
-      <c r="AF53" s="41"/>
-      <c r="AG53" s="41"/>
-      <c r="AH53" s="41"/>
-      <c r="AI53" s="41"/>
-      <c r="AJ53" s="41"/>
-      <c r="AK53" s="41"/>
-      <c r="AL53" s="41"/>
-      <c r="AM53" s="41"/>
-      <c r="AN53" s="41"/>
-      <c r="AO53" s="41"/>
+      <c r="T53" s="41">
+        <v>0.2</v>
+      </c>
+      <c r="U53" s="41">
+        <v>0.11</v>
+      </c>
+      <c r="V53" s="41">
+        <v>3.06</v>
+      </c>
+      <c r="W53" s="41">
+        <v>7.2729999999999997</v>
+      </c>
+      <c r="X53" s="41">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="Y53" s="41">
+        <v>49</v>
+      </c>
+      <c r="Z53" s="41">
+        <v>1.98</v>
+      </c>
+      <c r="AA53" s="41">
+        <v>140.9</v>
+      </c>
+      <c r="AB53" s="41">
+        <v>13.2</v>
+      </c>
+      <c r="AC53" s="41">
+        <v>28.3</v>
+      </c>
+      <c r="AD53" s="41">
+        <v>39.700000000000003</v>
+      </c>
+      <c r="AE53" s="17">
+        <v>7.2320000000000002</v>
+      </c>
+      <c r="AF53" s="41">
+        <v>411</v>
+      </c>
+      <c r="AG53" s="41">
+        <v>49.4</v>
+      </c>
+      <c r="AH53" s="41">
+        <v>7.2770000000000001</v>
+      </c>
+      <c r="AI53" s="41">
+        <v>34</v>
+      </c>
+      <c r="AJ53" s="41">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AK53" s="41">
+        <v>1.2</v>
+      </c>
+      <c r="AL53" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM53" s="41">
+        <v>12.3</v>
+      </c>
+      <c r="AN53" s="41">
+        <v>3.8</v>
+      </c>
+      <c r="AO53" s="41">
+        <v>198.5</v>
+      </c>
       <c r="AP53" s="74"/>
       <c r="AQ53" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.49399999999999999</v>
       </c>
       <c r="AR53" s="42">
         <f t="shared" si="50"/>
@@ -11835,11 +12764,11 @@
       </c>
       <c r="AS53" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>3.6000000000000014</v>
       </c>
       <c r="AT53" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>0.19999999999999973</v>
       </c>
       <c r="AU53" s="42">
         <f t="shared" si="57"/>
@@ -11867,23 +12796,23 @@
       <c r="BD53" s="22"/>
       <c r="BE53" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.6898702000000001E-3</v>
       </c>
       <c r="BF53" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.433413088</v>
       </c>
       <c r="BG53" s="43">
         <f t="shared" si="45"/>
-        <v>185.6</v>
-      </c>
-      <c r="BH53" s="44" t="str">
+        <v>198.5</v>
+      </c>
+      <c r="BH53" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI53" s="44" t="str">
+        <v>6.1964735516372799E-2</v>
+      </c>
+      <c r="BI53" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>6.1500000000000006E-2</v>
       </c>
       <c r="BJ53" s="44">
         <f t="shared" si="48"/>
@@ -11938,46 +12867,110 @@
       <c r="E54" s="40">
         <v>5</v>
       </c>
-      <c r="G54" s="35"/>
+      <c r="G54" s="35">
+        <v>45573.432638888888</v>
+      </c>
       <c r="H54" s="40">
         <v>2716.05</v>
       </c>
-      <c r="J54" s="41"/>
-      <c r="K54" s="41"/>
-      <c r="L54" s="41"/>
-      <c r="M54" s="41"/>
-      <c r="N54" s="41"/>
-      <c r="O54" s="41"/>
-      <c r="P54" s="41"/>
-      <c r="Q54" s="41"/>
-      <c r="R54" s="41"/>
+      <c r="J54" s="41">
+        <v>2546.25</v>
+      </c>
+      <c r="K54" s="41">
+        <v>24.582000000000001</v>
+      </c>
+      <c r="L54" s="41">
+        <v>23.151</v>
+      </c>
+      <c r="M54" s="41">
+        <v>94.2</v>
+      </c>
+      <c r="N54" s="41">
+        <v>16.29</v>
+      </c>
+      <c r="O54" s="41">
+        <v>333</v>
+      </c>
+      <c r="P54" s="41">
+        <v>1.32</v>
+      </c>
+      <c r="Q54" s="41">
+        <v>0.35</v>
+      </c>
+      <c r="R54" s="41">
+        <v>2.38</v>
+      </c>
       <c r="S54" s="41"/>
-      <c r="T54" s="41"/>
-      <c r="U54" s="41"/>
-      <c r="V54" s="41"/>
-      <c r="W54" s="41"/>
-      <c r="X54" s="41"/>
-      <c r="Y54" s="41"/>
-      <c r="Z54" s="41"/>
-      <c r="AA54" s="41"/>
-      <c r="AB54" s="41"/>
-      <c r="AC54" s="41"/>
-      <c r="AD54" s="41"/>
-      <c r="AE54" s="17"/>
-      <c r="AF54" s="41"/>
-      <c r="AG54" s="41"/>
-      <c r="AH54" s="41"/>
-      <c r="AI54" s="41"/>
-      <c r="AJ54" s="41"/>
-      <c r="AK54" s="41"/>
-      <c r="AL54" s="41"/>
-      <c r="AM54" s="41"/>
-      <c r="AN54" s="41"/>
-      <c r="AO54" s="41"/>
+      <c r="T54" s="41">
+        <v>0.19</v>
+      </c>
+      <c r="U54" s="41">
+        <v>0.13</v>
+      </c>
+      <c r="V54" s="41">
+        <v>3.08</v>
+      </c>
+      <c r="W54" s="41">
+        <v>7.2539999999999996</v>
+      </c>
+      <c r="X54" s="41">
+        <v>33.5</v>
+      </c>
+      <c r="Y54" s="41">
+        <v>54.6</v>
+      </c>
+      <c r="Z54" s="41">
+        <v>1.92</v>
+      </c>
+      <c r="AA54" s="41">
+        <v>142.19999999999999</v>
+      </c>
+      <c r="AB54" s="41">
+        <v>13.2</v>
+      </c>
+      <c r="AC54" s="41">
+        <v>29.5</v>
+      </c>
+      <c r="AD54" s="41">
+        <v>44.4</v>
+      </c>
+      <c r="AE54" s="17">
+        <v>7.2140000000000004</v>
+      </c>
+      <c r="AF54" s="41">
+        <v>411</v>
+      </c>
+      <c r="AG54" s="41">
+        <v>51.4</v>
+      </c>
+      <c r="AH54" s="41">
+        <v>7.3019999999999996</v>
+      </c>
+      <c r="AI54" s="41">
+        <v>34</v>
+      </c>
+      <c r="AJ54" s="41">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="AK54" s="41">
+        <v>1.7</v>
+      </c>
+      <c r="AL54" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM54" s="41">
+        <v>12.4</v>
+      </c>
+      <c r="AN54" s="41">
+        <v>4.2</v>
+      </c>
+      <c r="AO54" s="41">
+        <v>199.4</v>
+      </c>
       <c r="AP54" s="74"/>
       <c r="AQ54" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.51400000000000001</v>
       </c>
       <c r="AR54" s="42">
         <f t="shared" si="50"/>
@@ -11985,11 +12978,11 @@
       </c>
       <c r="AS54" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>3.9000000000000004</v>
       </c>
       <c r="AT54" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="AU54" s="42">
         <f t="shared" si="57"/>
@@ -12017,23 +13010,23 @@
       <c r="BD54" s="22"/>
       <c r="BE54" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.8465237600000001E-3</v>
       </c>
       <c r="BF54" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.6589942144000003</v>
       </c>
       <c r="BG54" s="43">
         <f t="shared" si="45"/>
-        <v>185.6</v>
-      </c>
-      <c r="BH54" s="44" t="str">
+        <v>199.4</v>
+      </c>
+      <c r="BH54" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI54" s="44" t="str">
+        <v>6.2186559679037114E-2</v>
+      </c>
+      <c r="BI54" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>6.2E-2</v>
       </c>
       <c r="BJ54" s="44">
         <f t="shared" si="48"/>
@@ -12088,54 +13081,118 @@
       <c r="E55" s="40">
         <v>5</v>
       </c>
-      <c r="G55" s="35"/>
+      <c r="G55" s="35">
+        <v>45573.437222222223</v>
+      </c>
       <c r="H55" s="40">
         <v>2716.05</v>
       </c>
-      <c r="J55" s="41"/>
-      <c r="K55" s="41"/>
-      <c r="L55" s="41"/>
-      <c r="M55" s="41"/>
-      <c r="N55" s="41"/>
-      <c r="O55" s="41"/>
-      <c r="P55" s="41"/>
-      <c r="Q55" s="41"/>
-      <c r="R55" s="41"/>
+      <c r="J55" s="41">
+        <v>2277.6750000000002</v>
+      </c>
+      <c r="K55" s="41">
+        <v>21.408999999999999</v>
+      </c>
+      <c r="L55" s="41">
+        <v>19.666</v>
+      </c>
+      <c r="M55" s="41">
+        <v>91.9</v>
+      </c>
+      <c r="N55" s="41">
+        <v>15.94</v>
+      </c>
+      <c r="O55" s="41">
+        <v>331</v>
+      </c>
+      <c r="P55" s="41">
+        <v>1.35</v>
+      </c>
+      <c r="Q55" s="41">
+        <v>0.39</v>
+      </c>
+      <c r="R55" s="41">
+        <v>1.77</v>
+      </c>
       <c r="S55" s="41"/>
-      <c r="T55" s="41"/>
-      <c r="U55" s="41"/>
-      <c r="V55" s="41"/>
-      <c r="W55" s="41"/>
-      <c r="X55" s="41"/>
-      <c r="Y55" s="41"/>
-      <c r="Z55" s="41"/>
-      <c r="AA55" s="41"/>
-      <c r="AB55" s="41"/>
-      <c r="AC55" s="41"/>
-      <c r="AD55" s="41"/>
-      <c r="AE55" s="17"/>
-      <c r="AF55" s="41"/>
-      <c r="AG55" s="41"/>
-      <c r="AH55" s="41"/>
-      <c r="AI55" s="41"/>
-      <c r="AJ55" s="41"/>
-      <c r="AK55" s="41"/>
-      <c r="AL55" s="41"/>
-      <c r="AM55" s="41"/>
-      <c r="AN55" s="41"/>
-      <c r="AO55" s="41"/>
+      <c r="T55" s="41">
+        <v>0.16</v>
+      </c>
+      <c r="U55" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="V55" s="41">
+        <v>3.43</v>
+      </c>
+      <c r="W55" s="41">
+        <v>7.2649999999999997</v>
+      </c>
+      <c r="X55" s="41">
+        <v>51.9</v>
+      </c>
+      <c r="Y55" s="41">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="Z55" s="41">
+        <v>2.6</v>
+      </c>
+      <c r="AA55" s="41">
+        <v>142.80000000000001</v>
+      </c>
+      <c r="AB55" s="41">
+        <v>20.9</v>
+      </c>
+      <c r="AC55" s="41">
+        <v>45.6</v>
+      </c>
+      <c r="AD55" s="41">
+        <v>55.2</v>
+      </c>
+      <c r="AE55" s="17">
+        <v>7.2240000000000002</v>
+      </c>
+      <c r="AF55" s="41">
+        <v>516</v>
+      </c>
+      <c r="AG55" s="41">
+        <v>52.2</v>
+      </c>
+      <c r="AH55" s="41">
+        <v>7.31</v>
+      </c>
+      <c r="AI55" s="41">
+        <v>34</v>
+      </c>
+      <c r="AJ55" s="41">
+        <v>2.6</v>
+      </c>
+      <c r="AK55" s="41">
+        <v>2.8</v>
+      </c>
+      <c r="AL55" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM55" s="41">
+        <v>7.7</v>
+      </c>
+      <c r="AN55" s="41">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AO55" s="41">
+        <v>198.1</v>
+      </c>
       <c r="AP55" s="74"/>
       <c r="AQ55" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.52200000000000002</v>
       </c>
       <c r="AR55" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>9.3500030400000003E-2</v>
       </c>
       <c r="AS55" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT55" s="42">
         <f t="shared" si="56"/>
@@ -12167,27 +13224,27 @@
       <c r="BD55" s="22"/>
       <c r="BE55" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.5583338400000002E-3</v>
       </c>
       <c r="BF55" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.2440007296000002</v>
       </c>
       <c r="BG55" s="43">
         <f t="shared" si="45"/>
-        <v>185.6</v>
-      </c>
-      <c r="BH55" s="44" t="str">
+        <v>198.1</v>
+      </c>
+      <c r="BH55" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI55" s="44" t="str">
+        <v>3.8869257950530034E-2</v>
+      </c>
+      <c r="BI55" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>3.85E-2</v>
       </c>
       <c r="BJ55" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>134.640043776</v>
       </c>
       <c r="BK55" s="44" t="str">
         <f t="shared" si="19"/>
@@ -12199,11 +13256,11 @@
       </c>
       <c r="BM55" s="45">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>9.3500030400000003E-2</v>
       </c>
       <c r="BN55" s="44">
         <f t="shared" si="58"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
       <c r="BO55" s="44" t="str">
         <f t="shared" si="49"/>
@@ -12211,15 +13268,15 @@
       </c>
       <c r="BP55" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>242.85722181818184</v>
       </c>
       <c r="BQ55" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>9.3500030400000003E-2</v>
       </c>
       <c r="BR55" s="24">
         <f t="shared" si="54"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:70" s="40" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -12238,54 +13295,118 @@
       <c r="E56" s="40">
         <v>5</v>
       </c>
-      <c r="G56" s="35"/>
+      <c r="G56" s="35">
+        <v>45573.441099537034</v>
+      </c>
       <c r="H56" s="40">
         <v>2716.05</v>
       </c>
-      <c r="J56" s="41"/>
-      <c r="K56" s="41"/>
-      <c r="L56" s="41"/>
-      <c r="M56" s="41"/>
-      <c r="N56" s="41"/>
-      <c r="O56" s="41"/>
-      <c r="P56" s="41"/>
-      <c r="Q56" s="41"/>
-      <c r="R56" s="41"/>
+      <c r="J56" s="41">
+        <v>2410.7399999999998</v>
+      </c>
+      <c r="K56" s="41">
+        <v>21.79</v>
+      </c>
+      <c r="L56" s="41">
+        <v>20.309999999999999</v>
+      </c>
+      <c r="M56" s="41">
+        <v>93.2</v>
+      </c>
+      <c r="N56" s="41">
+        <v>15.73</v>
+      </c>
+      <c r="O56" s="41">
+        <v>327</v>
+      </c>
+      <c r="P56" s="41">
+        <v>1.37</v>
+      </c>
+      <c r="Q56" s="41">
+        <v>0.37</v>
+      </c>
+      <c r="R56" s="41">
+        <v>2.14</v>
+      </c>
       <c r="S56" s="41"/>
-      <c r="T56" s="41"/>
-      <c r="U56" s="41"/>
-      <c r="V56" s="41"/>
-      <c r="W56" s="41"/>
-      <c r="X56" s="41"/>
-      <c r="Y56" s="41"/>
-      <c r="Z56" s="41"/>
-      <c r="AA56" s="41"/>
-      <c r="AB56" s="41"/>
-      <c r="AC56" s="41"/>
-      <c r="AD56" s="41"/>
-      <c r="AE56" s="17"/>
-      <c r="AF56" s="41"/>
-      <c r="AG56" s="41"/>
-      <c r="AH56" s="41"/>
-      <c r="AI56" s="41"/>
-      <c r="AJ56" s="41"/>
-      <c r="AK56" s="41"/>
-      <c r="AL56" s="41"/>
-      <c r="AM56" s="41"/>
-      <c r="AN56" s="41"/>
-      <c r="AO56" s="41"/>
+      <c r="T56" s="41">
+        <v>0.16</v>
+      </c>
+      <c r="U56" s="41">
+        <v>0.09</v>
+      </c>
+      <c r="V56" s="41">
+        <v>2.91</v>
+      </c>
+      <c r="W56" s="41">
+        <v>7.2750000000000004</v>
+      </c>
+      <c r="X56" s="41">
+        <v>47.4</v>
+      </c>
+      <c r="Y56" s="41">
+        <v>65.8</v>
+      </c>
+      <c r="Z56" s="41">
+        <v>2.63</v>
+      </c>
+      <c r="AA56" s="41">
+        <v>138.9</v>
+      </c>
+      <c r="AB56" s="41">
+        <v>19.5</v>
+      </c>
+      <c r="AC56" s="41">
+        <v>41.6</v>
+      </c>
+      <c r="AD56" s="41">
+        <v>53.7</v>
+      </c>
+      <c r="AE56" s="17">
+        <v>7.234</v>
+      </c>
+      <c r="AF56" s="41">
+        <v>406</v>
+      </c>
+      <c r="AG56" s="41">
+        <v>50.2</v>
+      </c>
+      <c r="AH56" s="41">
+        <v>7.3090000000000002</v>
+      </c>
+      <c r="AI56" s="41">
+        <v>34</v>
+      </c>
+      <c r="AJ56" s="41">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="AK56" s="41">
+        <v>2.8</v>
+      </c>
+      <c r="AL56" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AM56" s="41">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="AN56" s="41">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="AO56" s="41">
+        <v>197.8</v>
+      </c>
       <c r="AP56" s="75"/>
       <c r="AQ56" s="42">
         <f t="shared" si="43"/>
-        <v>0</v>
+        <v>0.502</v>
       </c>
       <c r="AR56" s="42">
         <f t="shared" si="50"/>
-        <v>0</v>
+        <v>9.6415632000000001E-2</v>
       </c>
       <c r="AS56" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>2.2999999999999989</v>
       </c>
       <c r="AT56" s="42">
         <f t="shared" si="56"/>
@@ -12317,27 +13438,27 @@
       <c r="BD56" s="22"/>
       <c r="BE56" s="43">
         <f t="shared" si="44"/>
-        <v>0</v>
+        <v>1.6069271999999998E-3</v>
       </c>
       <c r="BF56" s="43">
         <f t="shared" si="51"/>
-        <v>0</v>
+        <v>2.3139751679999994</v>
       </c>
       <c r="BG56" s="43">
         <f t="shared" si="45"/>
-        <v>185.6</v>
-      </c>
-      <c r="BH56" s="44" t="str">
+        <v>197.8</v>
+      </c>
+      <c r="BH56" s="44">
         <f t="shared" si="46"/>
-        <v/>
-      </c>
-      <c r="BI56" s="44" t="str">
+        <v>4.1456016177957529E-2</v>
+      </c>
+      <c r="BI56" s="44">
         <f t="shared" si="47"/>
-        <v/>
+        <v>4.0999999999999995E-2</v>
       </c>
       <c r="BJ56" s="44">
         <f t="shared" si="48"/>
-        <v>0</v>
+        <v>138.83851007999999</v>
       </c>
       <c r="BK56" s="44" t="str">
         <f t="shared" si="19"/>
@@ -12349,11 +13470,11 @@
       </c>
       <c r="BM56" s="45">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>9.6415632000000001E-2</v>
       </c>
       <c r="BN56" s="44">
         <f t="shared" si="58"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
       <c r="BO56" s="44" t="str">
         <f t="shared" si="49"/>
@@ -12361,15 +13482,15 @@
       </c>
       <c r="BP56" s="58">
         <f t="shared" si="52"/>
-        <v>0</v>
+        <v>250.43021298701299</v>
       </c>
       <c r="BQ56" s="46">
         <f t="shared" si="53"/>
-        <v>0</v>
+        <v>9.6415632000000001E-2</v>
       </c>
       <c r="BR56" s="24">
         <f t="shared" si="54"/>
-        <v>1.3919999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:70" s="40" customFormat="1" x14ac:dyDescent="0.3">
@@ -12437,11 +13558,11 @@
       </c>
       <c r="AS57" s="32">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-35159.5078125</v>
       </c>
       <c r="AT57" s="32">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-17535.712890625</v>
       </c>
       <c r="AU57" s="32">
         <f t="shared" si="57"/>
@@ -12588,11 +13709,11 @@
       </c>
       <c r="AS58" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-8.3000000000000007</v>
       </c>
       <c r="AT58" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="AU58" s="42">
         <f t="shared" si="57"/>
@@ -12739,11 +13860,11 @@
       </c>
       <c r="AS59" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-8.1999999999999993</v>
       </c>
       <c r="AT59" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-4.3</v>
       </c>
       <c r="AU59" s="42">
         <f t="shared" si="57"/>
@@ -12890,11 +14011,11 @@
       </c>
       <c r="AS60" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-11.3</v>
       </c>
       <c r="AT60" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-4.5</v>
       </c>
       <c r="AU60" s="42">
         <f t="shared" si="57"/>
@@ -13041,11 +14162,11 @@
       </c>
       <c r="AS61" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-11.7</v>
       </c>
       <c r="AT61" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-3.9</v>
       </c>
       <c r="AU61" s="42">
         <f t="shared" si="57"/>
@@ -13191,11 +14312,11 @@
       </c>
       <c r="AS62" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-12.3</v>
       </c>
       <c r="AT62" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-3.8</v>
       </c>
       <c r="AU62" s="42">
         <f t="shared" si="57"/>
@@ -13341,11 +14462,11 @@
       </c>
       <c r="AS63" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-12.4</v>
       </c>
       <c r="AT63" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-4.2</v>
       </c>
       <c r="AU63" s="42">
         <f t="shared" si="57"/>
@@ -13491,11 +14612,11 @@
       </c>
       <c r="AS64" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-7.7</v>
       </c>
       <c r="AT64" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-4.4000000000000004</v>
       </c>
       <c r="AU64" s="42">
         <f t="shared" si="57"/>
@@ -13641,11 +14762,11 @@
       </c>
       <c r="AS65" s="42">
         <f t="shared" si="55"/>
-        <v>0</v>
+        <v>-8.1999999999999993</v>
       </c>
       <c r="AT65" s="42">
         <f t="shared" si="56"/>
-        <v>0</v>
+        <v>-4.4000000000000004</v>
       </c>
       <c r="AU65" s="42">
         <f t="shared" si="57"/>
@@ -21477,33 +22598,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B75172DAFC2BB6479729CB287362C7E3" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0fc11b0946794a47057850b4f6c92dd7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34d8c884-fe7e-4d4f-a833-b92a2823f74b" xmlns:ns3="a198008e-c7f6-4ed0-9865-26ace3c97b59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb90ec7fe59ed1d44226abab88cd233b" ns2:_="" ns3:_="">
     <xsd:import namespace="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
@@ -21726,32 +22820,34 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F43DC28-AE43-4EFF-8739-4E0C557B415B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -21768,4 +22864,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
+    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>